<commit_message>
Restore master expense dataset and default workspace to master ledger
</commit_message>
<xml_diff>
--- a/expenses_data.xlsx
+++ b/expenses_data.xlsx
@@ -462,16 +462,16 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:G1"/>
+  <dimension ref="A1:G81"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="12" customWidth="1" min="1" max="1"/>
-    <col width="12" customWidth="1" min="2" max="2"/>
+    <col width="14" customWidth="1" min="2" max="2"/>
     <col width="14" customWidth="1" min="3" max="3"/>
-    <col width="12" customWidth="1" min="4" max="4"/>
+    <col width="27" customWidth="1" min="4" max="4"/>
     <col width="18" customWidth="1" min="5" max="5"/>
-    <col width="15" customWidth="1" min="6" max="6"/>
-    <col width="14" customWidth="1" min="7" max="7"/>
+    <col width="37" customWidth="1" min="6" max="6"/>
+    <col width="20" customWidth="1" min="7" max="7"/>
   </cols>
   <sheetData>
     <row r="1" ht="26" customHeight="1">
@@ -508,6 +508,2646 @@
       <c r="G1" s="1" t="inlineStr">
         <is>
           <t>Created At</t>
+        </is>
+      </c>
+    </row>
+    <row r="2">
+      <c r="A2" t="n">
+        <v>1</v>
+      </c>
+      <c r="B2" t="inlineStr">
+        <is>
+          <t>2026-07-25</t>
+        </is>
+      </c>
+      <c r="C2" t="n">
+        <v>22.6</v>
+      </c>
+      <c r="D2" t="inlineStr">
+        <is>
+          <t>Entertainment &amp; Leisure</t>
+        </is>
+      </c>
+      <c r="E2" t="inlineStr">
+        <is>
+          <t>Amex Card</t>
+        </is>
+      </c>
+      <c r="F2" t="inlineStr">
+        <is>
+          <t>Toronto Zoo</t>
+        </is>
+      </c>
+      <c r="G2" t="inlineStr">
+        <is>
+          <t>2026-08-14 00:04</t>
+        </is>
+      </c>
+    </row>
+    <row r="3">
+      <c r="A3" t="n">
+        <v>2</v>
+      </c>
+      <c r="B3" t="inlineStr">
+        <is>
+          <t>2026-07-25</t>
+        </is>
+      </c>
+      <c r="C3" t="n">
+        <v>20</v>
+      </c>
+      <c r="D3" t="inlineStr">
+        <is>
+          <t>Transportation</t>
+        </is>
+      </c>
+      <c r="E3" t="inlineStr">
+        <is>
+          <t>Amex Card</t>
+        </is>
+      </c>
+      <c r="F3" t="inlineStr">
+        <is>
+          <t>Petro-Canada</t>
+        </is>
+      </c>
+      <c r="G3" t="inlineStr">
+        <is>
+          <t>2026-08-14 00:04</t>
+        </is>
+      </c>
+    </row>
+    <row r="4">
+      <c r="A4" t="n">
+        <v>3</v>
+      </c>
+      <c r="B4" t="inlineStr">
+        <is>
+          <t>2026-07-24</t>
+        </is>
+      </c>
+      <c r="C4" t="n">
+        <v>26.6</v>
+      </c>
+      <c r="D4" t="inlineStr">
+        <is>
+          <t>Food &amp; Dining</t>
+        </is>
+      </c>
+      <c r="E4" t="inlineStr">
+        <is>
+          <t>Amex Card</t>
+        </is>
+      </c>
+      <c r="F4" t="inlineStr">
+        <is>
+          <t>Chaatter Box</t>
+        </is>
+      </c>
+      <c r="G4" t="inlineStr">
+        <is>
+          <t>2026-08-14 00:04</t>
+        </is>
+      </c>
+    </row>
+    <row r="5">
+      <c r="A5" t="n">
+        <v>4</v>
+      </c>
+      <c r="B5" t="inlineStr">
+        <is>
+          <t>2026-07-24</t>
+        </is>
+      </c>
+      <c r="C5" t="n">
+        <v>21.33</v>
+      </c>
+      <c r="D5" t="inlineStr">
+        <is>
+          <t>Shopping &amp; Retail</t>
+        </is>
+      </c>
+      <c r="E5" t="inlineStr">
+        <is>
+          <t>Amex Card</t>
+        </is>
+      </c>
+      <c r="F5" t="inlineStr">
+        <is>
+          <t>GoDirect Marketplace</t>
+        </is>
+      </c>
+      <c r="G5" t="inlineStr">
+        <is>
+          <t>2026-08-14 00:04</t>
+        </is>
+      </c>
+    </row>
+    <row r="6">
+      <c r="A6" t="n">
+        <v>5</v>
+      </c>
+      <c r="B6" t="inlineStr">
+        <is>
+          <t>2026-07-24</t>
+        </is>
+      </c>
+      <c r="C6" t="n">
+        <v>26.38</v>
+      </c>
+      <c r="D6" t="inlineStr">
+        <is>
+          <t>Food &amp; Dining</t>
+        </is>
+      </c>
+      <c r="E6" t="inlineStr">
+        <is>
+          <t>Amex Card</t>
+        </is>
+      </c>
+      <c r="F6" t="inlineStr">
+        <is>
+          <t>Zauq Restaurant</t>
+        </is>
+      </c>
+      <c r="G6" t="inlineStr">
+        <is>
+          <t>2026-08-14 00:04</t>
+        </is>
+      </c>
+    </row>
+    <row r="7">
+      <c r="A7" t="n">
+        <v>6</v>
+      </c>
+      <c r="B7" t="inlineStr">
+        <is>
+          <t>2026-07-24</t>
+        </is>
+      </c>
+      <c r="C7" t="n">
+        <v>26.38</v>
+      </c>
+      <c r="D7" t="inlineStr">
+        <is>
+          <t>Food &amp; Dining</t>
+        </is>
+      </c>
+      <c r="E7" t="inlineStr">
+        <is>
+          <t>Amex Card</t>
+        </is>
+      </c>
+      <c r="F7" t="inlineStr">
+        <is>
+          <t>Zauq Restaurant</t>
+        </is>
+      </c>
+      <c r="G7" t="inlineStr">
+        <is>
+          <t>2026-08-14 00:04</t>
+        </is>
+      </c>
+    </row>
+    <row r="8">
+      <c r="A8" t="n">
+        <v>7</v>
+      </c>
+      <c r="B8" t="inlineStr">
+        <is>
+          <t>2026-07-23</t>
+        </is>
+      </c>
+      <c r="C8" t="n">
+        <v>45.2</v>
+      </c>
+      <c r="D8" t="inlineStr">
+        <is>
+          <t>Shopping &amp; Retail</t>
+        </is>
+      </c>
+      <c r="E8" t="inlineStr">
+        <is>
+          <t>Amex Card</t>
+        </is>
+      </c>
+      <c r="F8" t="inlineStr">
+        <is>
+          <t>Banana Republic Factory</t>
+        </is>
+      </c>
+      <c r="G8" t="inlineStr">
+        <is>
+          <t>2026-08-14 00:04</t>
+        </is>
+      </c>
+    </row>
+    <row r="9">
+      <c r="A9" t="n">
+        <v>8</v>
+      </c>
+      <c r="B9" t="inlineStr">
+        <is>
+          <t>2026-07-23</t>
+        </is>
+      </c>
+      <c r="C9" t="n">
+        <v>83.17</v>
+      </c>
+      <c r="D9" t="inlineStr">
+        <is>
+          <t>Shopping &amp; Retail</t>
+        </is>
+      </c>
+      <c r="E9" t="inlineStr">
+        <is>
+          <t>Amex Card</t>
+        </is>
+      </c>
+      <c r="F9" t="inlineStr">
+        <is>
+          <t>Calvin Klein</t>
+        </is>
+      </c>
+      <c r="G9" t="inlineStr">
+        <is>
+          <t>2026-08-14 00:04</t>
+        </is>
+      </c>
+    </row>
+    <row r="10">
+      <c r="A10" t="n">
+        <v>9</v>
+      </c>
+      <c r="B10" t="inlineStr">
+        <is>
+          <t>2026-07-23</t>
+        </is>
+      </c>
+      <c r="C10" t="n">
+        <v>25.99</v>
+      </c>
+      <c r="D10" t="inlineStr">
+        <is>
+          <t>Food &amp; Dining</t>
+        </is>
+      </c>
+      <c r="E10" t="inlineStr">
+        <is>
+          <t>Amex Card</t>
+        </is>
+      </c>
+      <c r="F10" t="inlineStr">
+        <is>
+          <t>Chipotle Mexican Grill</t>
+        </is>
+      </c>
+      <c r="G10" t="inlineStr">
+        <is>
+          <t>2026-08-14 00:04</t>
+        </is>
+      </c>
+    </row>
+    <row r="11">
+      <c r="A11" t="n">
+        <v>10</v>
+      </c>
+      <c r="B11" t="inlineStr">
+        <is>
+          <t>2026-07-23</t>
+        </is>
+      </c>
+      <c r="C11" t="n">
+        <v>146.9</v>
+      </c>
+      <c r="D11" t="inlineStr">
+        <is>
+          <t>Shopping &amp; Retail</t>
+        </is>
+      </c>
+      <c r="E11" t="inlineStr">
+        <is>
+          <t>Amex Card</t>
+        </is>
+      </c>
+      <c r="F11" t="inlineStr">
+        <is>
+          <t>Puma</t>
+        </is>
+      </c>
+      <c r="G11" t="inlineStr">
+        <is>
+          <t>2026-08-14 00:04</t>
+        </is>
+      </c>
+    </row>
+    <row r="12">
+      <c r="A12" t="n">
+        <v>11</v>
+      </c>
+      <c r="B12" t="inlineStr">
+        <is>
+          <t>2026-07-23</t>
+        </is>
+      </c>
+      <c r="C12" t="n">
+        <v>4.5</v>
+      </c>
+      <c r="D12" t="inlineStr">
+        <is>
+          <t>Food &amp; Dining</t>
+        </is>
+      </c>
+      <c r="E12" t="inlineStr">
+        <is>
+          <t>Amex Card</t>
+        </is>
+      </c>
+      <c r="F12" t="inlineStr">
+        <is>
+          <t>Redhi Wale</t>
+        </is>
+      </c>
+      <c r="G12" t="inlineStr">
+        <is>
+          <t>2026-08-14 00:04</t>
+        </is>
+      </c>
+    </row>
+    <row r="13">
+      <c r="A13" t="n">
+        <v>12</v>
+      </c>
+      <c r="B13" t="inlineStr">
+        <is>
+          <t>2026-07-23</t>
+        </is>
+      </c>
+      <c r="C13" t="n">
+        <v>11.37</v>
+      </c>
+      <c r="D13" t="inlineStr">
+        <is>
+          <t>Transportation</t>
+        </is>
+      </c>
+      <c r="E13" t="inlineStr">
+        <is>
+          <t>Amex Card</t>
+        </is>
+      </c>
+      <c r="F13" t="inlineStr">
+        <is>
+          <t>Uber</t>
+        </is>
+      </c>
+      <c r="G13" t="inlineStr">
+        <is>
+          <t>2026-08-14 00:04</t>
+        </is>
+      </c>
+    </row>
+    <row r="14">
+      <c r="A14" t="n">
+        <v>13</v>
+      </c>
+      <c r="B14" t="inlineStr">
+        <is>
+          <t>2026-07-22</t>
+        </is>
+      </c>
+      <c r="C14" t="n">
+        <v>36.72</v>
+      </c>
+      <c r="D14" t="inlineStr">
+        <is>
+          <t>Entertainment &amp; Leisure</t>
+        </is>
+      </c>
+      <c r="E14" t="inlineStr">
+        <is>
+          <t>Amex Card</t>
+        </is>
+      </c>
+      <c r="F14" t="inlineStr">
+        <is>
+          <t>Cineplex</t>
+        </is>
+      </c>
+      <c r="G14" t="inlineStr">
+        <is>
+          <t>2026-08-14 00:04</t>
+        </is>
+      </c>
+    </row>
+    <row r="15">
+      <c r="A15" t="n">
+        <v>14</v>
+      </c>
+      <c r="B15" t="inlineStr">
+        <is>
+          <t>2026-07-22</t>
+        </is>
+      </c>
+      <c r="C15" t="n">
+        <v>9.890000000000001</v>
+      </c>
+      <c r="D15" t="inlineStr">
+        <is>
+          <t>Food &amp; Dining</t>
+        </is>
+      </c>
+      <c r="E15" t="inlineStr">
+        <is>
+          <t>Amex Card</t>
+        </is>
+      </c>
+      <c r="F15" t="inlineStr">
+        <is>
+          <t>Freshly Squeezed</t>
+        </is>
+      </c>
+      <c r="G15" t="inlineStr">
+        <is>
+          <t>2026-08-14 00:04</t>
+        </is>
+      </c>
+    </row>
+    <row r="16">
+      <c r="A16" t="n">
+        <v>15</v>
+      </c>
+      <c r="B16" t="inlineStr">
+        <is>
+          <t>2026-07-22</t>
+        </is>
+      </c>
+      <c r="C16" t="n">
+        <v>6.72</v>
+      </c>
+      <c r="D16" t="inlineStr">
+        <is>
+          <t>Food &amp; Dining</t>
+        </is>
+      </c>
+      <c r="E16" t="inlineStr">
+        <is>
+          <t>Amex Card</t>
+        </is>
+      </c>
+      <c r="F16" t="inlineStr">
+        <is>
+          <t>Mos Mos Bakery</t>
+        </is>
+      </c>
+      <c r="G16" t="inlineStr">
+        <is>
+          <t>2026-08-14 00:04</t>
+        </is>
+      </c>
+    </row>
+    <row r="17">
+      <c r="A17" t="n">
+        <v>16</v>
+      </c>
+      <c r="B17" t="inlineStr">
+        <is>
+          <t>2026-07-22</t>
+        </is>
+      </c>
+      <c r="C17" t="n">
+        <v>2.51</v>
+      </c>
+      <c r="D17" t="inlineStr">
+        <is>
+          <t>Food &amp; Dining</t>
+        </is>
+      </c>
+      <c r="E17" t="inlineStr">
+        <is>
+          <t>Amex Card</t>
+        </is>
+      </c>
+      <c r="F17" t="inlineStr">
+        <is>
+          <t>Patties Express</t>
+        </is>
+      </c>
+      <c r="G17" t="inlineStr">
+        <is>
+          <t>2026-08-14 00:04</t>
+        </is>
+      </c>
+    </row>
+    <row r="18">
+      <c r="A18" t="n">
+        <v>17</v>
+      </c>
+      <c r="B18" t="inlineStr">
+        <is>
+          <t>2026-07-22</t>
+        </is>
+      </c>
+      <c r="C18" t="n">
+        <v>6.6</v>
+      </c>
+      <c r="D18" t="inlineStr">
+        <is>
+          <t>Transportation</t>
+        </is>
+      </c>
+      <c r="E18" t="inlineStr">
+        <is>
+          <t>Amex Card</t>
+        </is>
+      </c>
+      <c r="F18" t="inlineStr">
+        <is>
+          <t>Presto</t>
+        </is>
+      </c>
+      <c r="G18" t="inlineStr">
+        <is>
+          <t>2026-08-14 00:04</t>
+        </is>
+      </c>
+    </row>
+    <row r="19">
+      <c r="A19" t="n">
+        <v>18</v>
+      </c>
+      <c r="B19" t="inlineStr">
+        <is>
+          <t>2026-07-22</t>
+        </is>
+      </c>
+      <c r="C19" t="n">
+        <v>19.21</v>
+      </c>
+      <c r="D19" t="inlineStr">
+        <is>
+          <t>Food &amp; Dining</t>
+        </is>
+      </c>
+      <c r="E19" t="inlineStr">
+        <is>
+          <t>Amex Card</t>
+        </is>
+      </c>
+      <c r="F19" t="inlineStr">
+        <is>
+          <t>Sultans Mediterranean Grill</t>
+        </is>
+      </c>
+      <c r="G19" t="inlineStr">
+        <is>
+          <t>2026-08-14 00:04</t>
+        </is>
+      </c>
+    </row>
+    <row r="20">
+      <c r="A20" t="n">
+        <v>19</v>
+      </c>
+      <c r="B20" t="inlineStr">
+        <is>
+          <t>2026-07-22</t>
+        </is>
+      </c>
+      <c r="C20" t="n">
+        <v>14.45</v>
+      </c>
+      <c r="D20" t="inlineStr">
+        <is>
+          <t>Food &amp; Dining</t>
+        </is>
+      </c>
+      <c r="E20" t="inlineStr">
+        <is>
+          <t>Amex Card</t>
+        </is>
+      </c>
+      <c r="F20" t="inlineStr">
+        <is>
+          <t>Sumaq Queen</t>
+        </is>
+      </c>
+      <c r="G20" t="inlineStr">
+        <is>
+          <t>2026-08-14 00:04</t>
+        </is>
+      </c>
+    </row>
+    <row r="21">
+      <c r="A21" t="n">
+        <v>20</v>
+      </c>
+      <c r="B21" t="inlineStr">
+        <is>
+          <t>2026-07-21</t>
+        </is>
+      </c>
+      <c r="C21" t="n">
+        <v>25.76</v>
+      </c>
+      <c r="D21" t="inlineStr">
+        <is>
+          <t>Food &amp; Dining</t>
+        </is>
+      </c>
+      <c r="E21" t="inlineStr">
+        <is>
+          <t>Amex Card</t>
+        </is>
+      </c>
+      <c r="F21" t="inlineStr">
+        <is>
+          <t>Uber Eats</t>
+        </is>
+      </c>
+      <c r="G21" t="inlineStr">
+        <is>
+          <t>2026-08-14 00:04</t>
+        </is>
+      </c>
+    </row>
+    <row r="22">
+      <c r="A22" t="n">
+        <v>21</v>
+      </c>
+      <c r="B22" t="inlineStr">
+        <is>
+          <t>2026-07-20</t>
+        </is>
+      </c>
+      <c r="C22" t="n">
+        <v>337.15</v>
+      </c>
+      <c r="D22" t="inlineStr">
+        <is>
+          <t>Shopping &amp; Retail</t>
+        </is>
+      </c>
+      <c r="E22" t="inlineStr">
+        <is>
+          <t>Amex Card</t>
+        </is>
+      </c>
+      <c r="F22" t="inlineStr">
+        <is>
+          <t>Mia Burton</t>
+        </is>
+      </c>
+      <c r="G22" t="inlineStr">
+        <is>
+          <t>2026-08-14 00:04</t>
+        </is>
+      </c>
+    </row>
+    <row r="23">
+      <c r="A23" t="n">
+        <v>22</v>
+      </c>
+      <c r="B23" t="inlineStr">
+        <is>
+          <t>2026-07-20</t>
+        </is>
+      </c>
+      <c r="C23" t="n">
+        <v>12.47</v>
+      </c>
+      <c r="D23" t="inlineStr">
+        <is>
+          <t>Food &amp; Dining</t>
+        </is>
+      </c>
+      <c r="E23" t="inlineStr">
+        <is>
+          <t>Amex Card</t>
+        </is>
+      </c>
+      <c r="F23" t="inlineStr">
+        <is>
+          <t>Nav's Grocery</t>
+        </is>
+      </c>
+      <c r="G23" t="inlineStr">
+        <is>
+          <t>2026-08-14 00:04</t>
+        </is>
+      </c>
+    </row>
+    <row r="24">
+      <c r="A24" t="n">
+        <v>23</v>
+      </c>
+      <c r="B24" t="inlineStr">
+        <is>
+          <t>2026-07-20</t>
+        </is>
+      </c>
+      <c r="C24" t="n">
+        <v>28.94</v>
+      </c>
+      <c r="D24" t="inlineStr">
+        <is>
+          <t>Transportation</t>
+        </is>
+      </c>
+      <c r="E24" t="inlineStr">
+        <is>
+          <t>Amex Card</t>
+        </is>
+      </c>
+      <c r="F24" t="inlineStr">
+        <is>
+          <t>Uber</t>
+        </is>
+      </c>
+      <c r="G24" t="inlineStr">
+        <is>
+          <t>2026-08-14 00:04</t>
+        </is>
+      </c>
+    </row>
+    <row r="25">
+      <c r="A25" t="n">
+        <v>24</v>
+      </c>
+      <c r="B25" t="inlineStr">
+        <is>
+          <t>2026-07-19</t>
+        </is>
+      </c>
+      <c r="C25" t="n">
+        <v>11.3</v>
+      </c>
+      <c r="D25" t="inlineStr">
+        <is>
+          <t>Food &amp; Dining</t>
+        </is>
+      </c>
+      <c r="E25" t="inlineStr">
+        <is>
+          <t>Amex Card</t>
+        </is>
+      </c>
+      <c r="F25" t="inlineStr">
+        <is>
+          <t>Fresh on Crawford</t>
+        </is>
+      </c>
+      <c r="G25" t="inlineStr">
+        <is>
+          <t>2026-08-14 00:04</t>
+        </is>
+      </c>
+    </row>
+    <row r="26">
+      <c r="A26" t="n">
+        <v>25</v>
+      </c>
+      <c r="B26" t="inlineStr">
+        <is>
+          <t>2026-07-19</t>
+        </is>
+      </c>
+      <c r="C26" t="n">
+        <v>32.08</v>
+      </c>
+      <c r="D26" t="inlineStr">
+        <is>
+          <t>Shopping &amp; Retail</t>
+        </is>
+      </c>
+      <c r="E26" t="inlineStr">
+        <is>
+          <t>Amex Card</t>
+        </is>
+      </c>
+      <c r="F26" t="inlineStr">
+        <is>
+          <t>GoDirect Marketplace</t>
+        </is>
+      </c>
+      <c r="G26" t="inlineStr">
+        <is>
+          <t>2026-08-14 00:04</t>
+        </is>
+      </c>
+    </row>
+    <row r="27">
+      <c r="A27" t="n">
+        <v>26</v>
+      </c>
+      <c r="B27" t="inlineStr">
+        <is>
+          <t>2026-07-19</t>
+        </is>
+      </c>
+      <c r="C27" t="n">
+        <v>117.34</v>
+      </c>
+      <c r="D27" t="inlineStr">
+        <is>
+          <t>Food &amp; Dining</t>
+        </is>
+      </c>
+      <c r="E27" t="inlineStr">
+        <is>
+          <t>Amex Card</t>
+        </is>
+      </c>
+      <c r="F27" t="inlineStr">
+        <is>
+          <t>Sunnys Chinese</t>
+        </is>
+      </c>
+      <c r="G27" t="inlineStr">
+        <is>
+          <t>2026-08-14 00:04</t>
+        </is>
+      </c>
+    </row>
+    <row r="28">
+      <c r="A28" t="n">
+        <v>27</v>
+      </c>
+      <c r="B28" t="inlineStr">
+        <is>
+          <t>2026-07-19</t>
+        </is>
+      </c>
+      <c r="C28" t="n">
+        <v>17.03</v>
+      </c>
+      <c r="D28" t="inlineStr">
+        <is>
+          <t>Food &amp; Dining</t>
+        </is>
+      </c>
+      <c r="E28" t="inlineStr">
+        <is>
+          <t>Amex Card</t>
+        </is>
+      </c>
+      <c r="F28" t="inlineStr">
+        <is>
+          <t>Roywoods</t>
+        </is>
+      </c>
+      <c r="G28" t="inlineStr">
+        <is>
+          <t>2026-08-14 00:04</t>
+        </is>
+      </c>
+    </row>
+    <row r="29">
+      <c r="A29" t="n">
+        <v>28</v>
+      </c>
+      <c r="B29" t="inlineStr">
+        <is>
+          <t>2026-07-18</t>
+        </is>
+      </c>
+      <c r="C29" t="n">
+        <v>23.73</v>
+      </c>
+      <c r="D29" t="inlineStr">
+        <is>
+          <t>Food &amp; Dining</t>
+        </is>
+      </c>
+      <c r="E29" t="inlineStr">
+        <is>
+          <t>Amex Card</t>
+        </is>
+      </c>
+      <c r="F29" t="inlineStr">
+        <is>
+          <t>L'Avenue</t>
+        </is>
+      </c>
+      <c r="G29" t="inlineStr">
+        <is>
+          <t>2026-08-14 00:04</t>
+        </is>
+      </c>
+    </row>
+    <row r="30">
+      <c r="A30" t="n">
+        <v>29</v>
+      </c>
+      <c r="B30" t="inlineStr">
+        <is>
+          <t>2026-07-18</t>
+        </is>
+      </c>
+      <c r="C30" t="n">
+        <v>60.99</v>
+      </c>
+      <c r="D30" t="inlineStr">
+        <is>
+          <t>Shopping &amp; Retail</t>
+        </is>
+      </c>
+      <c r="E30" t="inlineStr">
+        <is>
+          <t>Amex Card</t>
+        </is>
+      </c>
+      <c r="F30" t="inlineStr">
+        <is>
+          <t>Muji</t>
+        </is>
+      </c>
+      <c r="G30" t="inlineStr">
+        <is>
+          <t>2026-08-14 00:04</t>
+        </is>
+      </c>
+    </row>
+    <row r="31">
+      <c r="A31" t="n">
+        <v>30</v>
+      </c>
+      <c r="B31" t="inlineStr">
+        <is>
+          <t>2026-07-18</t>
+        </is>
+      </c>
+      <c r="C31" t="n">
+        <v>4.46</v>
+      </c>
+      <c r="D31" t="inlineStr">
+        <is>
+          <t>Food &amp; Dining</t>
+        </is>
+      </c>
+      <c r="E31" t="inlineStr">
+        <is>
+          <t>Amex Card</t>
+        </is>
+      </c>
+      <c r="F31" t="inlineStr">
+        <is>
+          <t>Uncle Tetsu's Japanese Cheesecake</t>
+        </is>
+      </c>
+      <c r="G31" t="inlineStr">
+        <is>
+          <t>2026-08-14 00:04</t>
+        </is>
+      </c>
+    </row>
+    <row r="32">
+      <c r="A32" t="n">
+        <v>31</v>
+      </c>
+      <c r="B32" t="inlineStr">
+        <is>
+          <t>2026-07-17</t>
+        </is>
+      </c>
+      <c r="C32" t="n">
+        <v>5.33</v>
+      </c>
+      <c r="D32" t="inlineStr">
+        <is>
+          <t>Food &amp; Dining</t>
+        </is>
+      </c>
+      <c r="E32" t="inlineStr">
+        <is>
+          <t>Amex Card</t>
+        </is>
+      </c>
+      <c r="F32" t="inlineStr">
+        <is>
+          <t>Island Cafe</t>
+        </is>
+      </c>
+      <c r="G32" t="inlineStr">
+        <is>
+          <t>2026-08-14 00:04</t>
+        </is>
+      </c>
+    </row>
+    <row r="33">
+      <c r="A33" t="n">
+        <v>32</v>
+      </c>
+      <c r="B33" t="inlineStr">
+        <is>
+          <t>2026-07-17</t>
+        </is>
+      </c>
+      <c r="C33" t="n">
+        <v>18.08</v>
+      </c>
+      <c r="D33" t="inlineStr">
+        <is>
+          <t>Food &amp; Dining</t>
+        </is>
+      </c>
+      <c r="E33" t="inlineStr">
+        <is>
+          <t>Amex Card</t>
+        </is>
+      </c>
+      <c r="F33" t="inlineStr">
+        <is>
+          <t>Mailo's</t>
+        </is>
+      </c>
+      <c r="G33" t="inlineStr">
+        <is>
+          <t>2026-08-14 00:04</t>
+        </is>
+      </c>
+    </row>
+    <row r="34">
+      <c r="A34" t="n">
+        <v>33</v>
+      </c>
+      <c r="B34" t="inlineStr">
+        <is>
+          <t>2026-07-15</t>
+        </is>
+      </c>
+      <c r="C34" t="n">
+        <v>6.72</v>
+      </c>
+      <c r="D34" t="inlineStr">
+        <is>
+          <t>Food &amp; Dining</t>
+        </is>
+      </c>
+      <c r="E34" t="inlineStr">
+        <is>
+          <t>Amex Card</t>
+        </is>
+      </c>
+      <c r="F34" t="inlineStr">
+        <is>
+          <t>Mos Mos Bakery</t>
+        </is>
+      </c>
+      <c r="G34" t="inlineStr">
+        <is>
+          <t>2026-08-14 00:04</t>
+        </is>
+      </c>
+    </row>
+    <row r="35">
+      <c r="A35" t="n">
+        <v>34</v>
+      </c>
+      <c r="B35" t="inlineStr">
+        <is>
+          <t>2026-07-15</t>
+        </is>
+      </c>
+      <c r="C35" t="n">
+        <v>2.64</v>
+      </c>
+      <c r="D35" t="inlineStr">
+        <is>
+          <t>Food &amp; Dining</t>
+        </is>
+      </c>
+      <c r="E35" t="inlineStr">
+        <is>
+          <t>Amex Card</t>
+        </is>
+      </c>
+      <c r="F35" t="inlineStr">
+        <is>
+          <t>Patties Express</t>
+        </is>
+      </c>
+      <c r="G35" t="inlineStr">
+        <is>
+          <t>2026-08-14 00:04</t>
+        </is>
+      </c>
+    </row>
+    <row r="36">
+      <c r="A36" t="n">
+        <v>35</v>
+      </c>
+      <c r="B36" t="inlineStr">
+        <is>
+          <t>2026-07-15</t>
+        </is>
+      </c>
+      <c r="C36" t="n">
+        <v>6.6</v>
+      </c>
+      <c r="D36" t="inlineStr">
+        <is>
+          <t>Transportation</t>
+        </is>
+      </c>
+      <c r="E36" t="inlineStr">
+        <is>
+          <t>Amex Card</t>
+        </is>
+      </c>
+      <c r="F36" t="inlineStr">
+        <is>
+          <t>Presto</t>
+        </is>
+      </c>
+      <c r="G36" t="inlineStr">
+        <is>
+          <t>2026-08-14 00:04</t>
+        </is>
+      </c>
+    </row>
+    <row r="37">
+      <c r="A37" t="n">
+        <v>36</v>
+      </c>
+      <c r="B37" t="inlineStr">
+        <is>
+          <t>2026-07-15</t>
+        </is>
+      </c>
+      <c r="C37" t="n">
+        <v>7.91</v>
+      </c>
+      <c r="D37" t="inlineStr">
+        <is>
+          <t>Food &amp; Dining</t>
+        </is>
+      </c>
+      <c r="E37" t="inlineStr">
+        <is>
+          <t>Amex Card</t>
+        </is>
+      </c>
+      <c r="F37" t="inlineStr">
+        <is>
+          <t>Zen Kyoto</t>
+        </is>
+      </c>
+      <c r="G37" t="inlineStr">
+        <is>
+          <t>2026-08-14 00:04</t>
+        </is>
+      </c>
+    </row>
+    <row r="38">
+      <c r="A38" t="n">
+        <v>37</v>
+      </c>
+      <c r="B38" t="inlineStr">
+        <is>
+          <t>2026-07-14</t>
+        </is>
+      </c>
+      <c r="C38" t="n">
+        <v>38.15</v>
+      </c>
+      <c r="D38" t="inlineStr">
+        <is>
+          <t>Utilities &amp; Bills</t>
+        </is>
+      </c>
+      <c r="E38" t="inlineStr">
+        <is>
+          <t>Amex Card</t>
+        </is>
+      </c>
+      <c r="F38" t="inlineStr">
+        <is>
+          <t>Aviva General Insurance</t>
+        </is>
+      </c>
+      <c r="G38" t="inlineStr">
+        <is>
+          <t>2026-08-14 00:04</t>
+        </is>
+      </c>
+    </row>
+    <row r="39">
+      <c r="A39" t="n">
+        <v>38</v>
+      </c>
+      <c r="B39" t="inlineStr">
+        <is>
+          <t>2026-07-14</t>
+        </is>
+      </c>
+      <c r="C39" t="n">
+        <v>25.98</v>
+      </c>
+      <c r="D39" t="inlineStr">
+        <is>
+          <t>Food &amp; Dining</t>
+        </is>
+      </c>
+      <c r="E39" t="inlineStr">
+        <is>
+          <t>Amex Card</t>
+        </is>
+      </c>
+      <c r="F39" t="inlineStr">
+        <is>
+          <t>Domino's Pizza</t>
+        </is>
+      </c>
+      <c r="G39" t="inlineStr">
+        <is>
+          <t>2026-08-14 00:04</t>
+        </is>
+      </c>
+    </row>
+    <row r="40">
+      <c r="A40" t="n">
+        <v>39</v>
+      </c>
+      <c r="B40" t="inlineStr">
+        <is>
+          <t>2026-07-13</t>
+        </is>
+      </c>
+      <c r="C40" t="n">
+        <v>31.63</v>
+      </c>
+      <c r="D40" t="inlineStr">
+        <is>
+          <t>Shopping &amp; Retail</t>
+        </is>
+      </c>
+      <c r="E40" t="inlineStr">
+        <is>
+          <t>Amex Card</t>
+        </is>
+      </c>
+      <c r="F40" t="inlineStr">
+        <is>
+          <t>Amazon</t>
+        </is>
+      </c>
+      <c r="G40" t="inlineStr">
+        <is>
+          <t>2026-08-14 00:04</t>
+        </is>
+      </c>
+    </row>
+    <row r="41">
+      <c r="A41" t="n">
+        <v>40</v>
+      </c>
+      <c r="B41" t="inlineStr">
+        <is>
+          <t>2026-07-13</t>
+        </is>
+      </c>
+      <c r="C41" t="n">
+        <v>13.56</v>
+      </c>
+      <c r="D41" t="inlineStr">
+        <is>
+          <t>Food &amp; Dining</t>
+        </is>
+      </c>
+      <c r="E41" t="inlineStr">
+        <is>
+          <t>Amex Card</t>
+        </is>
+      </c>
+      <c r="F41" t="inlineStr">
+        <is>
+          <t>La Diperie</t>
+        </is>
+      </c>
+      <c r="G41" t="inlineStr">
+        <is>
+          <t>2026-08-14 00:04</t>
+        </is>
+      </c>
+    </row>
+    <row r="42">
+      <c r="A42" t="n">
+        <v>41</v>
+      </c>
+      <c r="B42" t="inlineStr">
+        <is>
+          <t>2026-07-12</t>
+        </is>
+      </c>
+      <c r="C42" t="n">
+        <v>11.65</v>
+      </c>
+      <c r="D42" t="inlineStr">
+        <is>
+          <t>Shopping &amp; Retail</t>
+        </is>
+      </c>
+      <c r="E42" t="inlineStr">
+        <is>
+          <t>Amex Card</t>
+        </is>
+      </c>
+      <c r="F42" t="inlineStr">
+        <is>
+          <t>Amazon</t>
+        </is>
+      </c>
+      <c r="G42" t="inlineStr">
+        <is>
+          <t>2026-08-14 00:04</t>
+        </is>
+      </c>
+    </row>
+    <row r="43">
+      <c r="A43" t="n">
+        <v>42</v>
+      </c>
+      <c r="B43" t="inlineStr">
+        <is>
+          <t>2026-07-12</t>
+        </is>
+      </c>
+      <c r="C43" t="n">
+        <v>45.96</v>
+      </c>
+      <c r="D43" t="inlineStr">
+        <is>
+          <t>Food &amp; Dining</t>
+        </is>
+      </c>
+      <c r="E43" t="inlineStr">
+        <is>
+          <t>Amex Card</t>
+        </is>
+      </c>
+      <c r="F43" t="inlineStr">
+        <is>
+          <t>Domino's Pizza</t>
+        </is>
+      </c>
+      <c r="G43" t="inlineStr">
+        <is>
+          <t>2026-08-14 00:04</t>
+        </is>
+      </c>
+    </row>
+    <row r="44">
+      <c r="A44" t="n">
+        <v>43</v>
+      </c>
+      <c r="B44" t="inlineStr">
+        <is>
+          <t>2026-07-11</t>
+        </is>
+      </c>
+      <c r="C44" t="n">
+        <v>29.88</v>
+      </c>
+      <c r="D44" t="inlineStr">
+        <is>
+          <t>Food &amp; Dining</t>
+        </is>
+      </c>
+      <c r="E44" t="inlineStr">
+        <is>
+          <t>Amex Card</t>
+        </is>
+      </c>
+      <c r="F44" t="inlineStr">
+        <is>
+          <t>McDonald's</t>
+        </is>
+      </c>
+      <c r="G44" t="inlineStr">
+        <is>
+          <t>2026-08-14 00:04</t>
+        </is>
+      </c>
+    </row>
+    <row r="45">
+      <c r="A45" t="n">
+        <v>44</v>
+      </c>
+      <c r="B45" t="inlineStr">
+        <is>
+          <t>2026-07-11</t>
+        </is>
+      </c>
+      <c r="C45" t="n">
+        <v>5.24</v>
+      </c>
+      <c r="D45" t="inlineStr">
+        <is>
+          <t>Food &amp; Dining</t>
+        </is>
+      </c>
+      <c r="E45" t="inlineStr">
+        <is>
+          <t>Amex Card</t>
+        </is>
+      </c>
+      <c r="F45" t="inlineStr">
+        <is>
+          <t>Mount Molson Dairy Bar</t>
+        </is>
+      </c>
+      <c r="G45" t="inlineStr">
+        <is>
+          <t>2026-08-14 00:04</t>
+        </is>
+      </c>
+    </row>
+    <row r="46">
+      <c r="A46" t="n">
+        <v>45</v>
+      </c>
+      <c r="B46" t="inlineStr">
+        <is>
+          <t>2026-07-10</t>
+        </is>
+      </c>
+      <c r="C46" t="n">
+        <v>40.38</v>
+      </c>
+      <c r="D46" t="inlineStr">
+        <is>
+          <t>Food &amp; Dining</t>
+        </is>
+      </c>
+      <c r="E46" t="inlineStr">
+        <is>
+          <t>Amex Card</t>
+        </is>
+      </c>
+      <c r="F46" t="inlineStr">
+        <is>
+          <t>Domino's Pizza</t>
+        </is>
+      </c>
+      <c r="G46" t="inlineStr">
+        <is>
+          <t>2026-08-14 00:04</t>
+        </is>
+      </c>
+    </row>
+    <row r="47">
+      <c r="A47" t="n">
+        <v>46</v>
+      </c>
+      <c r="B47" t="inlineStr">
+        <is>
+          <t>2026-07-10</t>
+        </is>
+      </c>
+      <c r="C47" t="n">
+        <v>3.15</v>
+      </c>
+      <c r="D47" t="inlineStr">
+        <is>
+          <t>Food &amp; Dining</t>
+        </is>
+      </c>
+      <c r="E47" t="inlineStr">
+        <is>
+          <t>Amex Card</t>
+        </is>
+      </c>
+      <c r="F47" t="inlineStr">
+        <is>
+          <t>McDonald's</t>
+        </is>
+      </c>
+      <c r="G47" t="inlineStr">
+        <is>
+          <t>2026-08-14 00:04</t>
+        </is>
+      </c>
+    </row>
+    <row r="48">
+      <c r="A48" t="n">
+        <v>47</v>
+      </c>
+      <c r="B48" t="inlineStr">
+        <is>
+          <t>2026-07-10</t>
+        </is>
+      </c>
+      <c r="C48" t="n">
+        <v>18.16</v>
+      </c>
+      <c r="D48" t="inlineStr">
+        <is>
+          <t>Food &amp; Dining</t>
+        </is>
+      </c>
+      <c r="E48" t="inlineStr">
+        <is>
+          <t>Amex Card</t>
+        </is>
+      </c>
+      <c r="F48" t="inlineStr">
+        <is>
+          <t>McDonald's</t>
+        </is>
+      </c>
+      <c r="G48" t="inlineStr">
+        <is>
+          <t>2026-08-14 00:04</t>
+        </is>
+      </c>
+    </row>
+    <row r="49">
+      <c r="A49" t="n">
+        <v>48</v>
+      </c>
+      <c r="B49" t="inlineStr">
+        <is>
+          <t>2026-07-10</t>
+        </is>
+      </c>
+      <c r="C49" t="n">
+        <v>20.54</v>
+      </c>
+      <c r="D49" t="inlineStr">
+        <is>
+          <t>Shopping &amp; Retail</t>
+        </is>
+      </c>
+      <c r="E49" t="inlineStr">
+        <is>
+          <t>Amex Card</t>
+        </is>
+      </c>
+      <c r="F49" t="inlineStr">
+        <is>
+          <t>Walmart</t>
+        </is>
+      </c>
+      <c r="G49" t="inlineStr">
+        <is>
+          <t>2026-08-14 00:04</t>
+        </is>
+      </c>
+    </row>
+    <row r="50">
+      <c r="A50" t="n">
+        <v>49</v>
+      </c>
+      <c r="B50" t="inlineStr">
+        <is>
+          <t>2026-07-09</t>
+        </is>
+      </c>
+      <c r="C50" t="n">
+        <v>22.2</v>
+      </c>
+      <c r="D50" t="inlineStr">
+        <is>
+          <t>Food &amp; Dining</t>
+        </is>
+      </c>
+      <c r="E50" t="inlineStr">
+        <is>
+          <t>Amex Card</t>
+        </is>
+      </c>
+      <c r="F50" t="inlineStr">
+        <is>
+          <t>Chipotle Mexican Grill</t>
+        </is>
+      </c>
+      <c r="G50" t="inlineStr">
+        <is>
+          <t>2026-08-14 00:04</t>
+        </is>
+      </c>
+    </row>
+    <row r="51">
+      <c r="A51" t="n">
+        <v>50</v>
+      </c>
+      <c r="B51" t="inlineStr">
+        <is>
+          <t>2026-07-08</t>
+        </is>
+      </c>
+      <c r="C51" t="n">
+        <v>6.72</v>
+      </c>
+      <c r="D51" t="inlineStr">
+        <is>
+          <t>Food &amp; Dining</t>
+        </is>
+      </c>
+      <c r="E51" t="inlineStr">
+        <is>
+          <t>Amex Card</t>
+        </is>
+      </c>
+      <c r="F51" t="inlineStr">
+        <is>
+          <t>Mos Mos Bakery</t>
+        </is>
+      </c>
+      <c r="G51" t="inlineStr">
+        <is>
+          <t>2026-08-14 00:04</t>
+        </is>
+      </c>
+    </row>
+    <row r="52">
+      <c r="A52" t="n">
+        <v>51</v>
+      </c>
+      <c r="B52" t="inlineStr">
+        <is>
+          <t>2026-07-08</t>
+        </is>
+      </c>
+      <c r="C52" t="n">
+        <v>2.51</v>
+      </c>
+      <c r="D52" t="inlineStr">
+        <is>
+          <t>Food &amp; Dining</t>
+        </is>
+      </c>
+      <c r="E52" t="inlineStr">
+        <is>
+          <t>Amex Card</t>
+        </is>
+      </c>
+      <c r="F52" t="inlineStr">
+        <is>
+          <t>Patties Express</t>
+        </is>
+      </c>
+      <c r="G52" t="inlineStr">
+        <is>
+          <t>2026-08-14 00:04</t>
+        </is>
+      </c>
+    </row>
+    <row r="53">
+      <c r="A53" t="n">
+        <v>52</v>
+      </c>
+      <c r="B53" t="inlineStr">
+        <is>
+          <t>2026-07-08</t>
+        </is>
+      </c>
+      <c r="C53" t="n">
+        <v>6.6</v>
+      </c>
+      <c r="D53" t="inlineStr">
+        <is>
+          <t>Transportation</t>
+        </is>
+      </c>
+      <c r="E53" t="inlineStr">
+        <is>
+          <t>Amex Card</t>
+        </is>
+      </c>
+      <c r="F53" t="inlineStr">
+        <is>
+          <t>Presto</t>
+        </is>
+      </c>
+      <c r="G53" t="inlineStr">
+        <is>
+          <t>2026-08-14 00:04</t>
+        </is>
+      </c>
+    </row>
+    <row r="54">
+      <c r="A54" t="n">
+        <v>53</v>
+      </c>
+      <c r="B54" t="inlineStr">
+        <is>
+          <t>2026-07-08</t>
+        </is>
+      </c>
+      <c r="C54" t="n">
+        <v>19.21</v>
+      </c>
+      <c r="D54" t="inlineStr">
+        <is>
+          <t>Food &amp; Dining</t>
+        </is>
+      </c>
+      <c r="E54" t="inlineStr">
+        <is>
+          <t>Amex Card</t>
+        </is>
+      </c>
+      <c r="F54" t="inlineStr">
+        <is>
+          <t>Sultans Mediterranean Grill</t>
+        </is>
+      </c>
+      <c r="G54" t="inlineStr">
+        <is>
+          <t>2026-08-14 00:04</t>
+        </is>
+      </c>
+    </row>
+    <row r="55">
+      <c r="A55" t="n">
+        <v>54</v>
+      </c>
+      <c r="B55" t="inlineStr">
+        <is>
+          <t>2026-07-07</t>
+        </is>
+      </c>
+      <c r="C55" t="n">
+        <v>78.3</v>
+      </c>
+      <c r="D55" t="inlineStr">
+        <is>
+          <t>Shopping &amp; Retail</t>
+        </is>
+      </c>
+      <c r="E55" t="inlineStr">
+        <is>
+          <t>Amex Card</t>
+        </is>
+      </c>
+      <c r="F55" t="inlineStr">
+        <is>
+          <t>Amazon</t>
+        </is>
+      </c>
+      <c r="G55" t="inlineStr">
+        <is>
+          <t>2026-08-14 00:04</t>
+        </is>
+      </c>
+    </row>
+    <row r="56">
+      <c r="A56" t="n">
+        <v>55</v>
+      </c>
+      <c r="B56" t="inlineStr">
+        <is>
+          <t>2026-07-07</t>
+        </is>
+      </c>
+      <c r="C56" t="n">
+        <v>8.359999999999999</v>
+      </c>
+      <c r="D56" t="inlineStr">
+        <is>
+          <t>Transportation</t>
+        </is>
+      </c>
+      <c r="E56" t="inlineStr">
+        <is>
+          <t>Amex Card</t>
+        </is>
+      </c>
+      <c r="F56" t="inlineStr">
+        <is>
+          <t>Lyft</t>
+        </is>
+      </c>
+      <c r="G56" t="inlineStr">
+        <is>
+          <t>2026-08-14 00:04</t>
+        </is>
+      </c>
+    </row>
+    <row r="57">
+      <c r="A57" t="n">
+        <v>56</v>
+      </c>
+      <c r="B57" t="inlineStr">
+        <is>
+          <t>2026-07-07</t>
+        </is>
+      </c>
+      <c r="C57" t="n">
+        <v>6.72</v>
+      </c>
+      <c r="D57" t="inlineStr">
+        <is>
+          <t>Food &amp; Dining</t>
+        </is>
+      </c>
+      <c r="E57" t="inlineStr">
+        <is>
+          <t>Amex Card</t>
+        </is>
+      </c>
+      <c r="F57" t="inlineStr">
+        <is>
+          <t>Mos Mos Bakery</t>
+        </is>
+      </c>
+      <c r="G57" t="inlineStr">
+        <is>
+          <t>2026-08-14 00:04</t>
+        </is>
+      </c>
+    </row>
+    <row r="58">
+      <c r="A58" t="n">
+        <v>57</v>
+      </c>
+      <c r="B58" t="inlineStr">
+        <is>
+          <t>2026-07-07</t>
+        </is>
+      </c>
+      <c r="C58" t="n">
+        <v>5.02</v>
+      </c>
+      <c r="D58" t="inlineStr">
+        <is>
+          <t>Food &amp; Dining</t>
+        </is>
+      </c>
+      <c r="E58" t="inlineStr">
+        <is>
+          <t>Amex Card</t>
+        </is>
+      </c>
+      <c r="F58" t="inlineStr">
+        <is>
+          <t>Patties Express</t>
+        </is>
+      </c>
+      <c r="G58" t="inlineStr">
+        <is>
+          <t>2026-08-14 00:04</t>
+        </is>
+      </c>
+    </row>
+    <row r="59">
+      <c r="A59" t="n">
+        <v>58</v>
+      </c>
+      <c r="B59" t="inlineStr">
+        <is>
+          <t>2026-07-07</t>
+        </is>
+      </c>
+      <c r="C59" t="n">
+        <v>3.3</v>
+      </c>
+      <c r="D59" t="inlineStr">
+        <is>
+          <t>Transportation</t>
+        </is>
+      </c>
+      <c r="E59" t="inlineStr">
+        <is>
+          <t>Amex Card</t>
+        </is>
+      </c>
+      <c r="F59" t="inlineStr">
+        <is>
+          <t>Presto</t>
+        </is>
+      </c>
+      <c r="G59" t="inlineStr">
+        <is>
+          <t>2026-08-14 00:04</t>
+        </is>
+      </c>
+    </row>
+    <row r="60">
+      <c r="A60" t="n">
+        <v>59</v>
+      </c>
+      <c r="B60" t="inlineStr">
+        <is>
+          <t>2026-07-07</t>
+        </is>
+      </c>
+      <c r="C60" t="n">
+        <v>158.2</v>
+      </c>
+      <c r="D60" t="inlineStr">
+        <is>
+          <t>Shopping &amp; Retail</t>
+        </is>
+      </c>
+      <c r="E60" t="inlineStr">
+        <is>
+          <t>Amex Card</t>
+        </is>
+      </c>
+      <c r="F60" t="inlineStr">
+        <is>
+          <t>JD Sports</t>
+        </is>
+      </c>
+      <c r="G60" t="inlineStr">
+        <is>
+          <t>2026-08-14 00:04</t>
+        </is>
+      </c>
+    </row>
+    <row r="61">
+      <c r="A61" t="n">
+        <v>60</v>
+      </c>
+      <c r="B61" t="inlineStr">
+        <is>
+          <t>2026-07-07</t>
+        </is>
+      </c>
+      <c r="C61" t="n">
+        <v>21.71</v>
+      </c>
+      <c r="D61" t="inlineStr">
+        <is>
+          <t>Transportation</t>
+        </is>
+      </c>
+      <c r="E61" t="inlineStr">
+        <is>
+          <t>Amex Card</t>
+        </is>
+      </c>
+      <c r="F61" t="inlineStr">
+        <is>
+          <t>Union Station Toronto</t>
+        </is>
+      </c>
+      <c r="G61" t="inlineStr">
+        <is>
+          <t>2026-08-14 00:04</t>
+        </is>
+      </c>
+    </row>
+    <row r="62">
+      <c r="A62" t="n">
+        <v>61</v>
+      </c>
+      <c r="B62" t="inlineStr">
+        <is>
+          <t>2026-07-07</t>
+        </is>
+      </c>
+      <c r="C62" t="n">
+        <v>39.14</v>
+      </c>
+      <c r="D62" t="inlineStr">
+        <is>
+          <t>Food &amp; Dining</t>
+        </is>
+      </c>
+      <c r="E62" t="inlineStr">
+        <is>
+          <t>Amex Card</t>
+        </is>
+      </c>
+      <c r="F62" t="inlineStr">
+        <is>
+          <t>Uber Eats</t>
+        </is>
+      </c>
+      <c r="G62" t="inlineStr">
+        <is>
+          <t>2026-08-14 00:04</t>
+        </is>
+      </c>
+    </row>
+    <row r="63">
+      <c r="A63" t="n">
+        <v>62</v>
+      </c>
+      <c r="B63" t="inlineStr">
+        <is>
+          <t>2026-07-07</t>
+        </is>
+      </c>
+      <c r="C63" t="n">
+        <v>38.39</v>
+      </c>
+      <c r="D63" t="inlineStr">
+        <is>
+          <t>Shopping &amp; Retail</t>
+        </is>
+      </c>
+      <c r="E63" t="inlineStr">
+        <is>
+          <t>Amex Card</t>
+        </is>
+      </c>
+      <c r="F63" t="inlineStr">
+        <is>
+          <t>Winners</t>
+        </is>
+      </c>
+      <c r="G63" t="inlineStr">
+        <is>
+          <t>2026-08-14 00:04</t>
+        </is>
+      </c>
+    </row>
+    <row r="64">
+      <c r="A64" t="n">
+        <v>63</v>
+      </c>
+      <c r="B64" t="inlineStr">
+        <is>
+          <t>2026-07-05</t>
+        </is>
+      </c>
+      <c r="C64" t="n">
+        <v>63.39</v>
+      </c>
+      <c r="D64" t="inlineStr">
+        <is>
+          <t>Food &amp; Dining</t>
+        </is>
+      </c>
+      <c r="E64" t="inlineStr">
+        <is>
+          <t>Amex Card</t>
+        </is>
+      </c>
+      <c r="F64" t="inlineStr">
+        <is>
+          <t>JOEY King Street</t>
+        </is>
+      </c>
+      <c r="G64" t="inlineStr">
+        <is>
+          <t>2026-08-14 00:04</t>
+        </is>
+      </c>
+    </row>
+    <row r="65">
+      <c r="A65" t="n">
+        <v>64</v>
+      </c>
+      <c r="B65" t="inlineStr">
+        <is>
+          <t>2026-07-05</t>
+        </is>
+      </c>
+      <c r="C65" t="n">
+        <v>14.75</v>
+      </c>
+      <c r="D65" t="inlineStr">
+        <is>
+          <t>Food &amp; Dining</t>
+        </is>
+      </c>
+      <c r="E65" t="inlineStr">
+        <is>
+          <t>Amex Card</t>
+        </is>
+      </c>
+      <c r="F65" t="inlineStr">
+        <is>
+          <t>Uncle Tetsu's Japanese Cheesecake</t>
+        </is>
+      </c>
+      <c r="G65" t="inlineStr">
+        <is>
+          <t>2026-08-14 00:04</t>
+        </is>
+      </c>
+    </row>
+    <row r="66">
+      <c r="A66" t="n">
+        <v>65</v>
+      </c>
+      <c r="B66" t="inlineStr">
+        <is>
+          <t>2026-07-04</t>
+        </is>
+      </c>
+      <c r="C66" t="n">
+        <v>55.94</v>
+      </c>
+      <c r="D66" t="inlineStr">
+        <is>
+          <t>Entertainment &amp; Leisure</t>
+        </is>
+      </c>
+      <c r="E66" t="inlineStr">
+        <is>
+          <t>Amex Card</t>
+        </is>
+      </c>
+      <c r="F66" t="inlineStr">
+        <is>
+          <t>Cineplex</t>
+        </is>
+      </c>
+      <c r="G66" t="inlineStr">
+        <is>
+          <t>2026-08-14 00:04</t>
+        </is>
+      </c>
+    </row>
+    <row r="67">
+      <c r="A67" t="n">
+        <v>66</v>
+      </c>
+      <c r="B67" t="inlineStr">
+        <is>
+          <t>2026-07-04</t>
+        </is>
+      </c>
+      <c r="C67" t="n">
+        <v>20.57</v>
+      </c>
+      <c r="D67" t="inlineStr">
+        <is>
+          <t>Food &amp; Dining</t>
+        </is>
+      </c>
+      <c r="E67" t="inlineStr">
+        <is>
+          <t>Amex Card</t>
+        </is>
+      </c>
+      <c r="F67" t="inlineStr">
+        <is>
+          <t>Uber Eats</t>
+        </is>
+      </c>
+      <c r="G67" t="inlineStr">
+        <is>
+          <t>2026-08-14 00:04</t>
+        </is>
+      </c>
+    </row>
+    <row r="68">
+      <c r="A68" t="n">
+        <v>67</v>
+      </c>
+      <c r="B68" t="inlineStr">
+        <is>
+          <t>2026-07-03</t>
+        </is>
+      </c>
+      <c r="C68" t="n">
+        <v>6.72</v>
+      </c>
+      <c r="D68" t="inlineStr">
+        <is>
+          <t>Food &amp; Dining</t>
+        </is>
+      </c>
+      <c r="E68" t="inlineStr">
+        <is>
+          <t>Amex Card</t>
+        </is>
+      </c>
+      <c r="F68" t="inlineStr">
+        <is>
+          <t>Mos Mos Bakery</t>
+        </is>
+      </c>
+      <c r="G68" t="inlineStr">
+        <is>
+          <t>2026-08-14 00:04</t>
+        </is>
+      </c>
+    </row>
+    <row r="69">
+      <c r="A69" t="n">
+        <v>68</v>
+      </c>
+      <c r="B69" t="inlineStr">
+        <is>
+          <t>2026-07-03</t>
+        </is>
+      </c>
+      <c r="C69" t="n">
+        <v>3.3</v>
+      </c>
+      <c r="D69" t="inlineStr">
+        <is>
+          <t>Transportation</t>
+        </is>
+      </c>
+      <c r="E69" t="inlineStr">
+        <is>
+          <t>Amex Card</t>
+        </is>
+      </c>
+      <c r="F69" t="inlineStr">
+        <is>
+          <t>Presto</t>
+        </is>
+      </c>
+      <c r="G69" t="inlineStr">
+        <is>
+          <t>2026-08-14 00:04</t>
+        </is>
+      </c>
+    </row>
+    <row r="70">
+      <c r="A70" t="n">
+        <v>69</v>
+      </c>
+      <c r="B70" t="inlineStr">
+        <is>
+          <t>2026-07-03</t>
+        </is>
+      </c>
+      <c r="C70" t="n">
+        <v>35.35</v>
+      </c>
+      <c r="D70" t="inlineStr">
+        <is>
+          <t>Food &amp; Dining</t>
+        </is>
+      </c>
+      <c r="E70" t="inlineStr">
+        <is>
+          <t>Amex Card</t>
+        </is>
+      </c>
+      <c r="F70" t="inlineStr">
+        <is>
+          <t>Uber Eats</t>
+        </is>
+      </c>
+      <c r="G70" t="inlineStr">
+        <is>
+          <t>2026-08-14 00:04</t>
+        </is>
+      </c>
+    </row>
+    <row r="71">
+      <c r="A71" t="n">
+        <v>70</v>
+      </c>
+      <c r="B71" t="inlineStr">
+        <is>
+          <t>2026-07-02</t>
+        </is>
+      </c>
+      <c r="C71" t="n">
+        <v>18.08</v>
+      </c>
+      <c r="D71" t="inlineStr">
+        <is>
+          <t>Food &amp; Dining</t>
+        </is>
+      </c>
+      <c r="E71" t="inlineStr">
+        <is>
+          <t>Amex Card</t>
+        </is>
+      </c>
+      <c r="F71" t="inlineStr">
+        <is>
+          <t>Mailo's</t>
+        </is>
+      </c>
+      <c r="G71" t="inlineStr">
+        <is>
+          <t>2026-08-14 00:04</t>
+        </is>
+      </c>
+    </row>
+    <row r="72">
+      <c r="A72" t="n">
+        <v>71</v>
+      </c>
+      <c r="B72" t="inlineStr">
+        <is>
+          <t>2026-06-30</t>
+        </is>
+      </c>
+      <c r="C72" t="n">
+        <v>1.46</v>
+      </c>
+      <c r="D72" t="inlineStr">
+        <is>
+          <t>Entertainment &amp; Leisure</t>
+        </is>
+      </c>
+      <c r="E72" t="inlineStr">
+        <is>
+          <t>Amex Card</t>
+        </is>
+      </c>
+      <c r="F72" t="inlineStr">
+        <is>
+          <t>Apple</t>
+        </is>
+      </c>
+      <c r="G72" t="inlineStr">
+        <is>
+          <t>2026-08-14 00:04</t>
+        </is>
+      </c>
+    </row>
+    <row r="73">
+      <c r="A73" t="n">
+        <v>72</v>
+      </c>
+      <c r="B73" t="inlineStr">
+        <is>
+          <t>2026-06-29</t>
+        </is>
+      </c>
+      <c r="C73" t="n">
+        <v>25.94</v>
+      </c>
+      <c r="D73" t="inlineStr">
+        <is>
+          <t>Food &amp; Dining</t>
+        </is>
+      </c>
+      <c r="E73" t="inlineStr">
+        <is>
+          <t>Amex Card</t>
+        </is>
+      </c>
+      <c r="F73" t="inlineStr">
+        <is>
+          <t>Dave's Hot Chicken</t>
+        </is>
+      </c>
+      <c r="G73" t="inlineStr">
+        <is>
+          <t>2026-08-14 00:04</t>
+        </is>
+      </c>
+    </row>
+    <row r="74">
+      <c r="A74" t="n">
+        <v>73</v>
+      </c>
+      <c r="B74" t="inlineStr">
+        <is>
+          <t>2026-06-29</t>
+        </is>
+      </c>
+      <c r="C74" t="n">
+        <v>2.51</v>
+      </c>
+      <c r="D74" t="inlineStr">
+        <is>
+          <t>Food &amp; Dining</t>
+        </is>
+      </c>
+      <c r="E74" t="inlineStr">
+        <is>
+          <t>Amex Card</t>
+        </is>
+      </c>
+      <c r="F74" t="inlineStr">
+        <is>
+          <t>Patties Express</t>
+        </is>
+      </c>
+      <c r="G74" t="inlineStr">
+        <is>
+          <t>2026-08-14 00:04</t>
+        </is>
+      </c>
+    </row>
+    <row r="75">
+      <c r="A75" t="n">
+        <v>74</v>
+      </c>
+      <c r="B75" t="inlineStr">
+        <is>
+          <t>2026-06-29</t>
+        </is>
+      </c>
+      <c r="C75" t="n">
+        <v>3.3</v>
+      </c>
+      <c r="D75" t="inlineStr">
+        <is>
+          <t>Transportation</t>
+        </is>
+      </c>
+      <c r="E75" t="inlineStr">
+        <is>
+          <t>Amex Card</t>
+        </is>
+      </c>
+      <c r="F75" t="inlineStr">
+        <is>
+          <t>Presto</t>
+        </is>
+      </c>
+      <c r="G75" t="inlineStr">
+        <is>
+          <t>2026-08-14 00:04</t>
+        </is>
+      </c>
+    </row>
+    <row r="76">
+      <c r="A76" t="n">
+        <v>75</v>
+      </c>
+      <c r="B76" t="inlineStr">
+        <is>
+          <t>2026-06-29</t>
+        </is>
+      </c>
+      <c r="C76" t="n">
+        <v>75.63</v>
+      </c>
+      <c r="D76" t="inlineStr">
+        <is>
+          <t>Shopping &amp; Retail</t>
+        </is>
+      </c>
+      <c r="E76" t="inlineStr">
+        <is>
+          <t>Amex Card</t>
+        </is>
+      </c>
+      <c r="F76" t="inlineStr">
+        <is>
+          <t>Walmart</t>
+        </is>
+      </c>
+      <c r="G76" t="inlineStr">
+        <is>
+          <t>2026-08-14 00:04</t>
+        </is>
+      </c>
+    </row>
+    <row r="77">
+      <c r="A77" t="n">
+        <v>76</v>
+      </c>
+      <c r="B77" t="inlineStr">
+        <is>
+          <t>2026-06-28</t>
+        </is>
+      </c>
+      <c r="C77" t="n">
+        <v>25.99</v>
+      </c>
+      <c r="D77" t="inlineStr">
+        <is>
+          <t>Food &amp; Dining</t>
+        </is>
+      </c>
+      <c r="E77" t="inlineStr">
+        <is>
+          <t>Amex Card</t>
+        </is>
+      </c>
+      <c r="F77" t="inlineStr">
+        <is>
+          <t>Chipotle Mexican Grill</t>
+        </is>
+      </c>
+      <c r="G77" t="inlineStr">
+        <is>
+          <t>2026-08-14 00:04</t>
+        </is>
+      </c>
+    </row>
+    <row r="78">
+      <c r="A78" t="n">
+        <v>77</v>
+      </c>
+      <c r="B78" t="inlineStr">
+        <is>
+          <t>2026-06-28</t>
+        </is>
+      </c>
+      <c r="C78" t="n">
+        <v>16.39</v>
+      </c>
+      <c r="D78" t="inlineStr">
+        <is>
+          <t>Food &amp; Dining</t>
+        </is>
+      </c>
+      <c r="E78" t="inlineStr">
+        <is>
+          <t>Amex Card</t>
+        </is>
+      </c>
+      <c r="F78" t="inlineStr">
+        <is>
+          <t>Prince Street Pizza</t>
+        </is>
+      </c>
+      <c r="G78" t="inlineStr">
+        <is>
+          <t>2026-08-14 00:04</t>
+        </is>
+      </c>
+    </row>
+    <row r="79">
+      <c r="A79" t="n">
+        <v>78</v>
+      </c>
+      <c r="B79" t="inlineStr">
+        <is>
+          <t>2026-06-27</t>
+        </is>
+      </c>
+      <c r="C79" t="n">
+        <v>7.97</v>
+      </c>
+      <c r="D79" t="inlineStr">
+        <is>
+          <t>Food &amp; Dining</t>
+        </is>
+      </c>
+      <c r="E79" t="inlineStr">
+        <is>
+          <t>Amex Card</t>
+        </is>
+      </c>
+      <c r="F79" t="inlineStr">
+        <is>
+          <t>Balzac's Coffee Roasters</t>
+        </is>
+      </c>
+      <c r="G79" t="inlineStr">
+        <is>
+          <t>2026-08-14 00:04</t>
+        </is>
+      </c>
+    </row>
+    <row r="80">
+      <c r="A80" t="n">
+        <v>79</v>
+      </c>
+      <c r="B80" t="inlineStr">
+        <is>
+          <t>2026-06-27</t>
+        </is>
+      </c>
+      <c r="C80" t="n">
+        <v>42.09</v>
+      </c>
+      <c r="D80" t="inlineStr">
+        <is>
+          <t>Shopping &amp; Retail</t>
+        </is>
+      </c>
+      <c r="E80" t="inlineStr">
+        <is>
+          <t>Amex Card</t>
+        </is>
+      </c>
+      <c r="F80" t="inlineStr">
+        <is>
+          <t>Dollarama</t>
+        </is>
+      </c>
+      <c r="G80" t="inlineStr">
+        <is>
+          <t>2026-08-14 00:04</t>
+        </is>
+      </c>
+    </row>
+    <row r="81">
+      <c r="A81" t="n">
+        <v>80</v>
+      </c>
+      <c r="B81" t="inlineStr">
+        <is>
+          <t>2026-06-26</t>
+        </is>
+      </c>
+      <c r="C81" t="n">
+        <v>18.08</v>
+      </c>
+      <c r="D81" t="inlineStr">
+        <is>
+          <t>Food &amp; Dining</t>
+        </is>
+      </c>
+      <c r="E81" t="inlineStr">
+        <is>
+          <t>Amex Card</t>
+        </is>
+      </c>
+      <c r="F81" t="inlineStr">
+        <is>
+          <t>Mailo's</t>
+        </is>
+      </c>
+      <c r="G81" t="inlineStr">
+        <is>
+          <t>2026-08-14 00:04</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Fix August source data, master Excel dataset, and Telegram bot workspace linking
</commit_message>
<xml_diff>
--- a/expenses_data.xlsx
+++ b/expenses_data.xlsx
@@ -462,7 +462,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:G81"/>
+  <dimension ref="A1:G96"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="12" customWidth="1" min="1" max="1"/>
@@ -470,7 +470,7 @@
     <col width="14" customWidth="1" min="3" max="3"/>
     <col width="27" customWidth="1" min="4" max="4"/>
     <col width="18" customWidth="1" min="5" max="5"/>
-    <col width="37" customWidth="1" min="6" max="6"/>
+    <col width="42" customWidth="1" min="6" max="6"/>
     <col width="20" customWidth="1" min="7" max="7"/>
   </cols>
   <sheetData>
@@ -517,30 +517,30 @@
       </c>
       <c r="B2" t="inlineStr">
         <is>
-          <t>2026-07-25</t>
+          <t>2026-08-14</t>
         </is>
       </c>
       <c r="C2" t="n">
-        <v>22.6</v>
+        <v>250</v>
       </c>
       <c r="D2" t="inlineStr">
         <is>
-          <t>Entertainment &amp; Leisure</t>
+          <t>Investments &amp; Savings</t>
         </is>
       </c>
       <c r="E2" t="inlineStr">
         <is>
-          <t>Amex Card</t>
+          <t>Bank Transfer</t>
         </is>
       </c>
       <c r="F2" t="inlineStr">
         <is>
-          <t>Toronto Zoo</t>
+          <t>Vanguard S&amp;P 500 ETF Auto-Deposit</t>
         </is>
       </c>
       <c r="G2" t="inlineStr">
         <is>
-          <t>2026-08-14 00:04</t>
+          <t>2026-08-14 09:00</t>
         </is>
       </c>
     </row>
@@ -550,30 +550,30 @@
       </c>
       <c r="B3" t="inlineStr">
         <is>
-          <t>2026-07-25</t>
+          <t>2026-08-14</t>
         </is>
       </c>
       <c r="C3" t="n">
-        <v>20</v>
+        <v>18.75</v>
       </c>
       <c r="D3" t="inlineStr">
         <is>
-          <t>Transportation</t>
+          <t>Food &amp; Dining</t>
         </is>
       </c>
       <c r="E3" t="inlineStr">
         <is>
-          <t>Amex Card</t>
+          <t>Apple Pay</t>
         </is>
       </c>
       <c r="F3" t="inlineStr">
         <is>
-          <t>Petro-Canada</t>
+          <t>Starbucks Coffee &amp; Pastry</t>
         </is>
       </c>
       <c r="G3" t="inlineStr">
         <is>
-          <t>2026-08-14 00:04</t>
+          <t>2026-08-14 08:30</t>
         </is>
       </c>
     </row>
@@ -583,30 +583,30 @@
       </c>
       <c r="B4" t="inlineStr">
         <is>
-          <t>2026-07-24</t>
+          <t>2026-08-13</t>
         </is>
       </c>
       <c r="C4" t="n">
-        <v>26.6</v>
+        <v>75</v>
       </c>
       <c r="D4" t="inlineStr">
         <is>
-          <t>Food &amp; Dining</t>
+          <t>Utilities &amp; Bills</t>
         </is>
       </c>
       <c r="E4" t="inlineStr">
         <is>
-          <t>Amex Card</t>
+          <t>Online</t>
         </is>
       </c>
       <c r="F4" t="inlineStr">
         <is>
-          <t>Chaatter Box</t>
+          <t>Bell High-Speed Fiber Internet</t>
         </is>
       </c>
       <c r="G4" t="inlineStr">
         <is>
-          <t>2026-08-14 00:04</t>
+          <t>2026-08-13 14:15</t>
         </is>
       </c>
     </row>
@@ -616,15 +616,15 @@
       </c>
       <c r="B5" t="inlineStr">
         <is>
-          <t>2026-07-24</t>
+          <t>2026-08-12</t>
         </is>
       </c>
       <c r="C5" t="n">
-        <v>21.33</v>
+        <v>41.2</v>
       </c>
       <c r="D5" t="inlineStr">
         <is>
-          <t>Shopping &amp; Retail</t>
+          <t>Food &amp; Dining</t>
         </is>
       </c>
       <c r="E5" t="inlineStr">
@@ -634,12 +634,12 @@
       </c>
       <c r="F5" t="inlineStr">
         <is>
-          <t>GoDirect Marketplace</t>
+          <t>Trader Joe's Groceries</t>
         </is>
       </c>
       <c r="G5" t="inlineStr">
         <is>
-          <t>2026-08-14 00:04</t>
+          <t>2026-08-12 18:20</t>
         </is>
       </c>
     </row>
@@ -649,30 +649,30 @@
       </c>
       <c r="B6" t="inlineStr">
         <is>
-          <t>2026-07-24</t>
+          <t>2026-08-11</t>
         </is>
       </c>
       <c r="C6" t="n">
-        <v>26.38</v>
+        <v>39.99</v>
       </c>
       <c r="D6" t="inlineStr">
         <is>
-          <t>Food &amp; Dining</t>
+          <t>Education &amp; Learning</t>
         </is>
       </c>
       <c r="E6" t="inlineStr">
         <is>
-          <t>Amex Card</t>
+          <t>Credit Card</t>
         </is>
       </c>
       <c r="F6" t="inlineStr">
         <is>
-          <t>Zauq Restaurant</t>
+          <t>Coursera Plus Annual Subscription</t>
         </is>
       </c>
       <c r="G6" t="inlineStr">
         <is>
-          <t>2026-08-14 00:04</t>
+          <t>2026-08-11 11:00</t>
         </is>
       </c>
     </row>
@@ -682,30 +682,30 @@
       </c>
       <c r="B7" t="inlineStr">
         <is>
-          <t>2026-07-24</t>
+          <t>2026-08-10</t>
         </is>
       </c>
       <c r="C7" t="n">
-        <v>26.38</v>
+        <v>18.5</v>
       </c>
       <c r="D7" t="inlineStr">
         <is>
-          <t>Food &amp; Dining</t>
+          <t>Transportation</t>
         </is>
       </c>
       <c r="E7" t="inlineStr">
         <is>
-          <t>Amex Card</t>
+          <t>Credit Card</t>
         </is>
       </c>
       <c r="F7" t="inlineStr">
         <is>
-          <t>Zauq Restaurant</t>
+          <t>Uber Ride to Downtown</t>
         </is>
       </c>
       <c r="G7" t="inlineStr">
         <is>
-          <t>2026-08-14 00:04</t>
+          <t>2026-08-10 20:45</t>
         </is>
       </c>
     </row>
@@ -715,11 +715,11 @@
       </c>
       <c r="B8" t="inlineStr">
         <is>
-          <t>2026-07-23</t>
+          <t>2026-08-09</t>
         </is>
       </c>
       <c r="C8" t="n">
-        <v>45.2</v>
+        <v>10.14</v>
       </c>
       <c r="D8" t="inlineStr">
         <is>
@@ -733,12 +733,12 @@
       </c>
       <c r="F8" t="inlineStr">
         <is>
-          <t>Banana Republic Factory</t>
+          <t>Walmart Delivery Pass Mississauga</t>
         </is>
       </c>
       <c r="G8" t="inlineStr">
         <is>
-          <t>2026-08-14 00:04</t>
+          <t>2026-08-09 13:16</t>
         </is>
       </c>
     </row>
@@ -748,15 +748,15 @@
       </c>
       <c r="B9" t="inlineStr">
         <is>
-          <t>2026-07-23</t>
+          <t>2026-08-08</t>
         </is>
       </c>
       <c r="C9" t="n">
-        <v>83.17</v>
+        <v>88.5</v>
       </c>
       <c r="D9" t="inlineStr">
         <is>
-          <t>Shopping &amp; Retail</t>
+          <t>Food &amp; Dining</t>
         </is>
       </c>
       <c r="E9" t="inlineStr">
@@ -766,12 +766,12 @@
       </c>
       <c r="F9" t="inlineStr">
         <is>
-          <t>Calvin Klein</t>
+          <t>Zauq Fine Dining Dinner</t>
         </is>
       </c>
       <c r="G9" t="inlineStr">
         <is>
-          <t>2026-08-14 00:04</t>
+          <t>2026-08-08 19:30</t>
         </is>
       </c>
     </row>
@@ -781,30 +781,30 @@
       </c>
       <c r="B10" t="inlineStr">
         <is>
-          <t>2026-07-23</t>
+          <t>2026-08-07</t>
         </is>
       </c>
       <c r="C10" t="n">
-        <v>25.99</v>
+        <v>45</v>
       </c>
       <c r="D10" t="inlineStr">
         <is>
-          <t>Food &amp; Dining</t>
+          <t>Personal Care</t>
         </is>
       </c>
       <c r="E10" t="inlineStr">
         <is>
-          <t>Amex Card</t>
+          <t>Cash</t>
         </is>
       </c>
       <c r="F10" t="inlineStr">
         <is>
-          <t>Chipotle Mexican Grill</t>
+          <t>Gentleman's Barber Club Haircut</t>
         </is>
       </c>
       <c r="G10" t="inlineStr">
         <is>
-          <t>2026-08-14 00:04</t>
+          <t>2026-08-07 16:00</t>
         </is>
       </c>
     </row>
@@ -814,30 +814,30 @@
       </c>
       <c r="B11" t="inlineStr">
         <is>
-          <t>2026-07-23</t>
+          <t>2026-08-06</t>
         </is>
       </c>
       <c r="C11" t="n">
-        <v>146.9</v>
+        <v>65</v>
       </c>
       <c r="D11" t="inlineStr">
         <is>
-          <t>Shopping &amp; Retail</t>
+          <t>Healthcare &amp; Wellness</t>
         </is>
       </c>
       <c r="E11" t="inlineStr">
         <is>
-          <t>Amex Card</t>
+          <t>Debit Card</t>
         </is>
       </c>
       <c r="F11" t="inlineStr">
         <is>
-          <t>Puma</t>
+          <t>Shoppers Drug Mart Vitamins &amp; Health</t>
         </is>
       </c>
       <c r="G11" t="inlineStr">
         <is>
-          <t>2026-08-14 00:04</t>
+          <t>2026-08-06 12:10</t>
         </is>
       </c>
     </row>
@@ -847,11 +847,11 @@
       </c>
       <c r="B12" t="inlineStr">
         <is>
-          <t>2026-07-23</t>
+          <t>2026-08-05</t>
         </is>
       </c>
       <c r="C12" t="n">
-        <v>4.5</v>
+        <v>32.45</v>
       </c>
       <c r="D12" t="inlineStr">
         <is>
@@ -860,17 +860,17 @@
       </c>
       <c r="E12" t="inlineStr">
         <is>
-          <t>Amex Card</t>
+          <t>Apple Pay</t>
         </is>
       </c>
       <c r="F12" t="inlineStr">
         <is>
-          <t>Redhi Wale</t>
+          <t>Chipotle Mexican Grill Bowl &amp; Drink</t>
         </is>
       </c>
       <c r="G12" t="inlineStr">
         <is>
-          <t>2026-08-14 00:04</t>
+          <t>2026-08-05 13:00</t>
         </is>
       </c>
     </row>
@@ -880,30 +880,30 @@
       </c>
       <c r="B13" t="inlineStr">
         <is>
-          <t>2026-07-23</t>
+          <t>2026-08-04</t>
         </is>
       </c>
       <c r="C13" t="n">
-        <v>11.37</v>
+        <v>24.99</v>
       </c>
       <c r="D13" t="inlineStr">
         <is>
-          <t>Transportation</t>
+          <t>Entertainment &amp; Leisure</t>
         </is>
       </c>
       <c r="E13" t="inlineStr">
         <is>
-          <t>Amex Card</t>
+          <t>Credit Card</t>
         </is>
       </c>
       <c r="F13" t="inlineStr">
         <is>
-          <t>Uber</t>
+          <t>Netflix 4K Ultra &amp; Spotify Bundle</t>
         </is>
       </c>
       <c r="G13" t="inlineStr">
         <is>
-          <t>2026-08-14 00:04</t>
+          <t>2026-08-04 10:00</t>
         </is>
       </c>
     </row>
@@ -913,30 +913,30 @@
       </c>
       <c r="B14" t="inlineStr">
         <is>
-          <t>2026-07-22</t>
+          <t>2026-08-03</t>
         </is>
       </c>
       <c r="C14" t="n">
-        <v>36.72</v>
+        <v>52</v>
       </c>
       <c r="D14" t="inlineStr">
         <is>
-          <t>Entertainment &amp; Leisure</t>
+          <t>Transportation</t>
         </is>
       </c>
       <c r="E14" t="inlineStr">
         <is>
-          <t>Amex Card</t>
+          <t>Credit Card</t>
         </is>
       </c>
       <c r="F14" t="inlineStr">
         <is>
-          <t>Cineplex</t>
+          <t>Shell Gas Station Refuel</t>
         </is>
       </c>
       <c r="G14" t="inlineStr">
         <is>
-          <t>2026-08-14 00:04</t>
+          <t>2026-08-03 17:45</t>
         </is>
       </c>
     </row>
@@ -946,11 +946,11 @@
       </c>
       <c r="B15" t="inlineStr">
         <is>
-          <t>2026-07-22</t>
+          <t>2026-08-02</t>
         </is>
       </c>
       <c r="C15" t="n">
-        <v>9.890000000000001</v>
+        <v>64.8</v>
       </c>
       <c r="D15" t="inlineStr">
         <is>
@@ -964,12 +964,12 @@
       </c>
       <c r="F15" t="inlineStr">
         <is>
-          <t>Freshly Squeezed</t>
+          <t>Whole Foods Market Organic Groceries</t>
         </is>
       </c>
       <c r="G15" t="inlineStr">
         <is>
-          <t>2026-08-14 00:04</t>
+          <t>2026-08-02 15:20</t>
         </is>
       </c>
     </row>
@@ -979,30 +979,30 @@
       </c>
       <c r="B16" t="inlineStr">
         <is>
-          <t>2026-07-22</t>
+          <t>2026-08-01</t>
         </is>
       </c>
       <c r="C16" t="n">
-        <v>6.72</v>
+        <v>115.4</v>
       </c>
       <c r="D16" t="inlineStr">
         <is>
-          <t>Food &amp; Dining</t>
+          <t>Utilities &amp; Bills</t>
         </is>
       </c>
       <c r="E16" t="inlineStr">
         <is>
-          <t>Amex Card</t>
+          <t>Online</t>
         </is>
       </c>
       <c r="F16" t="inlineStr">
         <is>
-          <t>Mos Mos Bakery</t>
+          <t>Hydro &amp; Electricity Monthly Bill</t>
         </is>
       </c>
       <c r="G16" t="inlineStr">
         <is>
-          <t>2026-08-14 00:04</t>
+          <t>2026-08-01 10:30</t>
         </is>
       </c>
     </row>
@@ -1012,30 +1012,30 @@
       </c>
       <c r="B17" t="inlineStr">
         <is>
-          <t>2026-07-22</t>
+          <t>2026-08-01</t>
         </is>
       </c>
       <c r="C17" t="n">
-        <v>2.51</v>
+        <v>1450</v>
       </c>
       <c r="D17" t="inlineStr">
         <is>
-          <t>Food &amp; Dining</t>
+          <t>Housing &amp; Rent</t>
         </is>
       </c>
       <c r="E17" t="inlineStr">
         <is>
-          <t>Amex Card</t>
+          <t>Bank Transfer</t>
         </is>
       </c>
       <c r="F17" t="inlineStr">
         <is>
-          <t>Patties Express</t>
+          <t>Downtown Luxury Apartment Monthly Rent</t>
         </is>
       </c>
       <c r="G17" t="inlineStr">
         <is>
-          <t>2026-08-14 00:04</t>
+          <t>2026-08-01 08:00</t>
         </is>
       </c>
     </row>
@@ -1045,15 +1045,15 @@
       </c>
       <c r="B18" t="inlineStr">
         <is>
-          <t>2026-07-22</t>
+          <t>2026-07-25</t>
         </is>
       </c>
       <c r="C18" t="n">
-        <v>6.6</v>
+        <v>22.6</v>
       </c>
       <c r="D18" t="inlineStr">
         <is>
-          <t>Transportation</t>
+          <t>Entertainment &amp; Leisure</t>
         </is>
       </c>
       <c r="E18" t="inlineStr">
@@ -1063,7 +1063,7 @@
       </c>
       <c r="F18" t="inlineStr">
         <is>
-          <t>Presto</t>
+          <t>Toronto Zoo</t>
         </is>
       </c>
       <c r="G18" t="inlineStr">
@@ -1078,15 +1078,15 @@
       </c>
       <c r="B19" t="inlineStr">
         <is>
-          <t>2026-07-22</t>
+          <t>2026-07-25</t>
         </is>
       </c>
       <c r="C19" t="n">
-        <v>19.21</v>
+        <v>20</v>
       </c>
       <c r="D19" t="inlineStr">
         <is>
-          <t>Food &amp; Dining</t>
+          <t>Transportation</t>
         </is>
       </c>
       <c r="E19" t="inlineStr">
@@ -1096,7 +1096,7 @@
       </c>
       <c r="F19" t="inlineStr">
         <is>
-          <t>Sultans Mediterranean Grill</t>
+          <t>Petro-Canada</t>
         </is>
       </c>
       <c r="G19" t="inlineStr">
@@ -1111,11 +1111,11 @@
       </c>
       <c r="B20" t="inlineStr">
         <is>
-          <t>2026-07-22</t>
+          <t>2026-07-24</t>
         </is>
       </c>
       <c r="C20" t="n">
-        <v>14.45</v>
+        <v>26.6</v>
       </c>
       <c r="D20" t="inlineStr">
         <is>
@@ -1129,7 +1129,7 @@
       </c>
       <c r="F20" t="inlineStr">
         <is>
-          <t>Sumaq Queen</t>
+          <t>Chaatter Box</t>
         </is>
       </c>
       <c r="G20" t="inlineStr">
@@ -1144,15 +1144,15 @@
       </c>
       <c r="B21" t="inlineStr">
         <is>
-          <t>2026-07-21</t>
+          <t>2026-07-24</t>
         </is>
       </c>
       <c r="C21" t="n">
-        <v>25.76</v>
+        <v>21.33</v>
       </c>
       <c r="D21" t="inlineStr">
         <is>
-          <t>Food &amp; Dining</t>
+          <t>Shopping &amp; Retail</t>
         </is>
       </c>
       <c r="E21" t="inlineStr">
@@ -1162,7 +1162,7 @@
       </c>
       <c r="F21" t="inlineStr">
         <is>
-          <t>Uber Eats</t>
+          <t>GoDirect Marketplace</t>
         </is>
       </c>
       <c r="G21" t="inlineStr">
@@ -1177,15 +1177,15 @@
       </c>
       <c r="B22" t="inlineStr">
         <is>
-          <t>2026-07-20</t>
+          <t>2026-07-24</t>
         </is>
       </c>
       <c r="C22" t="n">
-        <v>337.15</v>
+        <v>26.38</v>
       </c>
       <c r="D22" t="inlineStr">
         <is>
-          <t>Shopping &amp; Retail</t>
+          <t>Food &amp; Dining</t>
         </is>
       </c>
       <c r="E22" t="inlineStr">
@@ -1195,7 +1195,7 @@
       </c>
       <c r="F22" t="inlineStr">
         <is>
-          <t>Mia Burton</t>
+          <t>Zauq Restaurant</t>
         </is>
       </c>
       <c r="G22" t="inlineStr">
@@ -1210,15 +1210,15 @@
       </c>
       <c r="B23" t="inlineStr">
         <is>
-          <t>2026-07-20</t>
+          <t>2026-07-23</t>
         </is>
       </c>
       <c r="C23" t="n">
-        <v>12.47</v>
+        <v>45.2</v>
       </c>
       <c r="D23" t="inlineStr">
         <is>
-          <t>Food &amp; Dining</t>
+          <t>Shopping &amp; Retail</t>
         </is>
       </c>
       <c r="E23" t="inlineStr">
@@ -1228,7 +1228,7 @@
       </c>
       <c r="F23" t="inlineStr">
         <is>
-          <t>Nav's Grocery</t>
+          <t>Banana Republic Factory</t>
         </is>
       </c>
       <c r="G23" t="inlineStr">
@@ -1243,15 +1243,15 @@
       </c>
       <c r="B24" t="inlineStr">
         <is>
-          <t>2026-07-20</t>
+          <t>2026-07-23</t>
         </is>
       </c>
       <c r="C24" t="n">
-        <v>28.94</v>
+        <v>83.17</v>
       </c>
       <c r="D24" t="inlineStr">
         <is>
-          <t>Transportation</t>
+          <t>Shopping &amp; Retail</t>
         </is>
       </c>
       <c r="E24" t="inlineStr">
@@ -1261,7 +1261,7 @@
       </c>
       <c r="F24" t="inlineStr">
         <is>
-          <t>Uber</t>
+          <t>Calvin Klein</t>
         </is>
       </c>
       <c r="G24" t="inlineStr">
@@ -1276,11 +1276,11 @@
       </c>
       <c r="B25" t="inlineStr">
         <is>
-          <t>2026-07-19</t>
+          <t>2026-07-23</t>
         </is>
       </c>
       <c r="C25" t="n">
-        <v>11.3</v>
+        <v>25.99</v>
       </c>
       <c r="D25" t="inlineStr">
         <is>
@@ -1294,7 +1294,7 @@
       </c>
       <c r="F25" t="inlineStr">
         <is>
-          <t>Fresh on Crawford</t>
+          <t>Chipotle Mexican Grill</t>
         </is>
       </c>
       <c r="G25" t="inlineStr">
@@ -1309,11 +1309,11 @@
       </c>
       <c r="B26" t="inlineStr">
         <is>
-          <t>2026-07-19</t>
+          <t>2026-07-23</t>
         </is>
       </c>
       <c r="C26" t="n">
-        <v>32.08</v>
+        <v>146.9</v>
       </c>
       <c r="D26" t="inlineStr">
         <is>
@@ -1327,7 +1327,7 @@
       </c>
       <c r="F26" t="inlineStr">
         <is>
-          <t>GoDirect Marketplace</t>
+          <t>Puma</t>
         </is>
       </c>
       <c r="G26" t="inlineStr">
@@ -1342,11 +1342,11 @@
       </c>
       <c r="B27" t="inlineStr">
         <is>
-          <t>2026-07-19</t>
+          <t>2026-07-23</t>
         </is>
       </c>
       <c r="C27" t="n">
-        <v>117.34</v>
+        <v>4.5</v>
       </c>
       <c r="D27" t="inlineStr">
         <is>
@@ -1360,7 +1360,7 @@
       </c>
       <c r="F27" t="inlineStr">
         <is>
-          <t>Sunnys Chinese</t>
+          <t>Redhi Wale</t>
         </is>
       </c>
       <c r="G27" t="inlineStr">
@@ -1375,15 +1375,15 @@
       </c>
       <c r="B28" t="inlineStr">
         <is>
-          <t>2026-07-19</t>
+          <t>2026-07-23</t>
         </is>
       </c>
       <c r="C28" t="n">
-        <v>17.03</v>
+        <v>11.37</v>
       </c>
       <c r="D28" t="inlineStr">
         <is>
-          <t>Food &amp; Dining</t>
+          <t>Transportation</t>
         </is>
       </c>
       <c r="E28" t="inlineStr">
@@ -1393,7 +1393,7 @@
       </c>
       <c r="F28" t="inlineStr">
         <is>
-          <t>Roywoods</t>
+          <t>Uber</t>
         </is>
       </c>
       <c r="G28" t="inlineStr">
@@ -1408,15 +1408,15 @@
       </c>
       <c r="B29" t="inlineStr">
         <is>
-          <t>2026-07-18</t>
+          <t>2026-07-22</t>
         </is>
       </c>
       <c r="C29" t="n">
-        <v>23.73</v>
+        <v>36.72</v>
       </c>
       <c r="D29" t="inlineStr">
         <is>
-          <t>Food &amp; Dining</t>
+          <t>Entertainment &amp; Leisure</t>
         </is>
       </c>
       <c r="E29" t="inlineStr">
@@ -1426,7 +1426,7 @@
       </c>
       <c r="F29" t="inlineStr">
         <is>
-          <t>L'Avenue</t>
+          <t>Cineplex</t>
         </is>
       </c>
       <c r="G29" t="inlineStr">
@@ -1441,15 +1441,15 @@
       </c>
       <c r="B30" t="inlineStr">
         <is>
-          <t>2026-07-18</t>
+          <t>2026-07-22</t>
         </is>
       </c>
       <c r="C30" t="n">
-        <v>60.99</v>
+        <v>9.890000000000001</v>
       </c>
       <c r="D30" t="inlineStr">
         <is>
-          <t>Shopping &amp; Retail</t>
+          <t>Food &amp; Dining</t>
         </is>
       </c>
       <c r="E30" t="inlineStr">
@@ -1459,7 +1459,7 @@
       </c>
       <c r="F30" t="inlineStr">
         <is>
-          <t>Muji</t>
+          <t>Freshly Squeezed</t>
         </is>
       </c>
       <c r="G30" t="inlineStr">
@@ -1474,11 +1474,11 @@
       </c>
       <c r="B31" t="inlineStr">
         <is>
-          <t>2026-07-18</t>
+          <t>2026-07-22</t>
         </is>
       </c>
       <c r="C31" t="n">
-        <v>4.46</v>
+        <v>6.72</v>
       </c>
       <c r="D31" t="inlineStr">
         <is>
@@ -1492,7 +1492,7 @@
       </c>
       <c r="F31" t="inlineStr">
         <is>
-          <t>Uncle Tetsu's Japanese Cheesecake</t>
+          <t>Mos Mos Bakery</t>
         </is>
       </c>
       <c r="G31" t="inlineStr">
@@ -1507,11 +1507,11 @@
       </c>
       <c r="B32" t="inlineStr">
         <is>
-          <t>2026-07-17</t>
+          <t>2026-07-22</t>
         </is>
       </c>
       <c r="C32" t="n">
-        <v>5.33</v>
+        <v>2.51</v>
       </c>
       <c r="D32" t="inlineStr">
         <is>
@@ -1525,7 +1525,7 @@
       </c>
       <c r="F32" t="inlineStr">
         <is>
-          <t>Island Cafe</t>
+          <t>Patties Express</t>
         </is>
       </c>
       <c r="G32" t="inlineStr">
@@ -1540,15 +1540,15 @@
       </c>
       <c r="B33" t="inlineStr">
         <is>
-          <t>2026-07-17</t>
+          <t>2026-07-22</t>
         </is>
       </c>
       <c r="C33" t="n">
-        <v>18.08</v>
+        <v>6.6</v>
       </c>
       <c r="D33" t="inlineStr">
         <is>
-          <t>Food &amp; Dining</t>
+          <t>Transportation</t>
         </is>
       </c>
       <c r="E33" t="inlineStr">
@@ -1558,7 +1558,7 @@
       </c>
       <c r="F33" t="inlineStr">
         <is>
-          <t>Mailo's</t>
+          <t>Presto</t>
         </is>
       </c>
       <c r="G33" t="inlineStr">
@@ -1573,11 +1573,11 @@
       </c>
       <c r="B34" t="inlineStr">
         <is>
-          <t>2026-07-15</t>
+          <t>2026-07-22</t>
         </is>
       </c>
       <c r="C34" t="n">
-        <v>6.72</v>
+        <v>19.21</v>
       </c>
       <c r="D34" t="inlineStr">
         <is>
@@ -1591,7 +1591,7 @@
       </c>
       <c r="F34" t="inlineStr">
         <is>
-          <t>Mos Mos Bakery</t>
+          <t>Sultans Mediterranean Grill</t>
         </is>
       </c>
       <c r="G34" t="inlineStr">
@@ -1606,11 +1606,11 @@
       </c>
       <c r="B35" t="inlineStr">
         <is>
-          <t>2026-07-15</t>
+          <t>2026-07-22</t>
         </is>
       </c>
       <c r="C35" t="n">
-        <v>2.64</v>
+        <v>14.45</v>
       </c>
       <c r="D35" t="inlineStr">
         <is>
@@ -1624,7 +1624,7 @@
       </c>
       <c r="F35" t="inlineStr">
         <is>
-          <t>Patties Express</t>
+          <t>Sumaq Queen</t>
         </is>
       </c>
       <c r="G35" t="inlineStr">
@@ -1639,15 +1639,15 @@
       </c>
       <c r="B36" t="inlineStr">
         <is>
-          <t>2026-07-15</t>
+          <t>2026-07-21</t>
         </is>
       </c>
       <c r="C36" t="n">
-        <v>6.6</v>
+        <v>25.76</v>
       </c>
       <c r="D36" t="inlineStr">
         <is>
-          <t>Transportation</t>
+          <t>Food &amp; Dining</t>
         </is>
       </c>
       <c r="E36" t="inlineStr">
@@ -1657,7 +1657,7 @@
       </c>
       <c r="F36" t="inlineStr">
         <is>
-          <t>Presto</t>
+          <t>Uber Eats</t>
         </is>
       </c>
       <c r="G36" t="inlineStr">
@@ -1672,15 +1672,15 @@
       </c>
       <c r="B37" t="inlineStr">
         <is>
-          <t>2026-07-15</t>
+          <t>2026-07-20</t>
         </is>
       </c>
       <c r="C37" t="n">
-        <v>7.91</v>
+        <v>337.15</v>
       </c>
       <c r="D37" t="inlineStr">
         <is>
-          <t>Food &amp; Dining</t>
+          <t>Shopping &amp; Retail</t>
         </is>
       </c>
       <c r="E37" t="inlineStr">
@@ -1690,7 +1690,7 @@
       </c>
       <c r="F37" t="inlineStr">
         <is>
-          <t>Zen Kyoto</t>
+          <t>Mia Burton</t>
         </is>
       </c>
       <c r="G37" t="inlineStr">
@@ -1705,15 +1705,15 @@
       </c>
       <c r="B38" t="inlineStr">
         <is>
-          <t>2026-07-14</t>
+          <t>2026-07-20</t>
         </is>
       </c>
       <c r="C38" t="n">
-        <v>38.15</v>
+        <v>12.47</v>
       </c>
       <c r="D38" t="inlineStr">
         <is>
-          <t>Utilities &amp; Bills</t>
+          <t>Food &amp; Dining</t>
         </is>
       </c>
       <c r="E38" t="inlineStr">
@@ -1723,7 +1723,7 @@
       </c>
       <c r="F38" t="inlineStr">
         <is>
-          <t>Aviva General Insurance</t>
+          <t>Nav's Grocery</t>
         </is>
       </c>
       <c r="G38" t="inlineStr">
@@ -1738,15 +1738,15 @@
       </c>
       <c r="B39" t="inlineStr">
         <is>
-          <t>2026-07-14</t>
+          <t>2026-07-20</t>
         </is>
       </c>
       <c r="C39" t="n">
-        <v>25.98</v>
+        <v>28.94</v>
       </c>
       <c r="D39" t="inlineStr">
         <is>
-          <t>Food &amp; Dining</t>
+          <t>Transportation</t>
         </is>
       </c>
       <c r="E39" t="inlineStr">
@@ -1756,7 +1756,7 @@
       </c>
       <c r="F39" t="inlineStr">
         <is>
-          <t>Domino's Pizza</t>
+          <t>Uber</t>
         </is>
       </c>
       <c r="G39" t="inlineStr">
@@ -1771,15 +1771,15 @@
       </c>
       <c r="B40" t="inlineStr">
         <is>
-          <t>2026-07-13</t>
+          <t>2026-07-19</t>
         </is>
       </c>
       <c r="C40" t="n">
-        <v>31.63</v>
+        <v>11.3</v>
       </c>
       <c r="D40" t="inlineStr">
         <is>
-          <t>Shopping &amp; Retail</t>
+          <t>Food &amp; Dining</t>
         </is>
       </c>
       <c r="E40" t="inlineStr">
@@ -1789,7 +1789,7 @@
       </c>
       <c r="F40" t="inlineStr">
         <is>
-          <t>Amazon</t>
+          <t>Fresh on Crawford</t>
         </is>
       </c>
       <c r="G40" t="inlineStr">
@@ -1804,15 +1804,15 @@
       </c>
       <c r="B41" t="inlineStr">
         <is>
-          <t>2026-07-13</t>
+          <t>2026-07-19</t>
         </is>
       </c>
       <c r="C41" t="n">
-        <v>13.56</v>
+        <v>32.08</v>
       </c>
       <c r="D41" t="inlineStr">
         <is>
-          <t>Food &amp; Dining</t>
+          <t>Shopping &amp; Retail</t>
         </is>
       </c>
       <c r="E41" t="inlineStr">
@@ -1822,7 +1822,7 @@
       </c>
       <c r="F41" t="inlineStr">
         <is>
-          <t>La Diperie</t>
+          <t>GoDirect Marketplace</t>
         </is>
       </c>
       <c r="G41" t="inlineStr">
@@ -1837,15 +1837,15 @@
       </c>
       <c r="B42" t="inlineStr">
         <is>
-          <t>2026-07-12</t>
+          <t>2026-07-19</t>
         </is>
       </c>
       <c r="C42" t="n">
-        <v>11.65</v>
+        <v>117.34</v>
       </c>
       <c r="D42" t="inlineStr">
         <is>
-          <t>Shopping &amp; Retail</t>
+          <t>Food &amp; Dining</t>
         </is>
       </c>
       <c r="E42" t="inlineStr">
@@ -1855,7 +1855,7 @@
       </c>
       <c r="F42" t="inlineStr">
         <is>
-          <t>Amazon</t>
+          <t>Sunnys Chinese</t>
         </is>
       </c>
       <c r="G42" t="inlineStr">
@@ -1870,11 +1870,11 @@
       </c>
       <c r="B43" t="inlineStr">
         <is>
-          <t>2026-07-12</t>
+          <t>2026-07-19</t>
         </is>
       </c>
       <c r="C43" t="n">
-        <v>45.96</v>
+        <v>17.03</v>
       </c>
       <c r="D43" t="inlineStr">
         <is>
@@ -1888,7 +1888,7 @@
       </c>
       <c r="F43" t="inlineStr">
         <is>
-          <t>Domino's Pizza</t>
+          <t>Roywoods</t>
         </is>
       </c>
       <c r="G43" t="inlineStr">
@@ -1903,11 +1903,11 @@
       </c>
       <c r="B44" t="inlineStr">
         <is>
-          <t>2026-07-11</t>
+          <t>2026-07-18</t>
         </is>
       </c>
       <c r="C44" t="n">
-        <v>29.88</v>
+        <v>23.73</v>
       </c>
       <c r="D44" t="inlineStr">
         <is>
@@ -1921,7 +1921,7 @@
       </c>
       <c r="F44" t="inlineStr">
         <is>
-          <t>McDonald's</t>
+          <t>L'Avenue</t>
         </is>
       </c>
       <c r="G44" t="inlineStr">
@@ -1936,15 +1936,15 @@
       </c>
       <c r="B45" t="inlineStr">
         <is>
-          <t>2026-07-11</t>
+          <t>2026-07-18</t>
         </is>
       </c>
       <c r="C45" t="n">
-        <v>5.24</v>
+        <v>60.99</v>
       </c>
       <c r="D45" t="inlineStr">
         <is>
-          <t>Food &amp; Dining</t>
+          <t>Shopping &amp; Retail</t>
         </is>
       </c>
       <c r="E45" t="inlineStr">
@@ -1954,7 +1954,7 @@
       </c>
       <c r="F45" t="inlineStr">
         <is>
-          <t>Mount Molson Dairy Bar</t>
+          <t>Muji</t>
         </is>
       </c>
       <c r="G45" t="inlineStr">
@@ -1969,11 +1969,11 @@
       </c>
       <c r="B46" t="inlineStr">
         <is>
-          <t>2026-07-10</t>
+          <t>2026-07-18</t>
         </is>
       </c>
       <c r="C46" t="n">
-        <v>40.38</v>
+        <v>4.46</v>
       </c>
       <c r="D46" t="inlineStr">
         <is>
@@ -1987,7 +1987,7 @@
       </c>
       <c r="F46" t="inlineStr">
         <is>
-          <t>Domino's Pizza</t>
+          <t>Uncle Tetsu's Japanese Cheesecake</t>
         </is>
       </c>
       <c r="G46" t="inlineStr">
@@ -2002,11 +2002,11 @@
       </c>
       <c r="B47" t="inlineStr">
         <is>
-          <t>2026-07-10</t>
+          <t>2026-07-17</t>
         </is>
       </c>
       <c r="C47" t="n">
-        <v>3.15</v>
+        <v>5.33</v>
       </c>
       <c r="D47" t="inlineStr">
         <is>
@@ -2020,7 +2020,7 @@
       </c>
       <c r="F47" t="inlineStr">
         <is>
-          <t>McDonald's</t>
+          <t>Island Cafe</t>
         </is>
       </c>
       <c r="G47" t="inlineStr">
@@ -2035,11 +2035,11 @@
       </c>
       <c r="B48" t="inlineStr">
         <is>
-          <t>2026-07-10</t>
+          <t>2026-07-17</t>
         </is>
       </c>
       <c r="C48" t="n">
-        <v>18.16</v>
+        <v>18.08</v>
       </c>
       <c r="D48" t="inlineStr">
         <is>
@@ -2053,7 +2053,7 @@
       </c>
       <c r="F48" t="inlineStr">
         <is>
-          <t>McDonald's</t>
+          <t>Mailo's</t>
         </is>
       </c>
       <c r="G48" t="inlineStr">
@@ -2068,15 +2068,15 @@
       </c>
       <c r="B49" t="inlineStr">
         <is>
-          <t>2026-07-10</t>
+          <t>2026-07-15</t>
         </is>
       </c>
       <c r="C49" t="n">
-        <v>20.54</v>
+        <v>6.72</v>
       </c>
       <c r="D49" t="inlineStr">
         <is>
-          <t>Shopping &amp; Retail</t>
+          <t>Food &amp; Dining</t>
         </is>
       </c>
       <c r="E49" t="inlineStr">
@@ -2086,7 +2086,7 @@
       </c>
       <c r="F49" t="inlineStr">
         <is>
-          <t>Walmart</t>
+          <t>Mos Mos Bakery</t>
         </is>
       </c>
       <c r="G49" t="inlineStr">
@@ -2101,11 +2101,11 @@
       </c>
       <c r="B50" t="inlineStr">
         <is>
-          <t>2026-07-09</t>
+          <t>2026-07-15</t>
         </is>
       </c>
       <c r="C50" t="n">
-        <v>22.2</v>
+        <v>2.64</v>
       </c>
       <c r="D50" t="inlineStr">
         <is>
@@ -2119,7 +2119,7 @@
       </c>
       <c r="F50" t="inlineStr">
         <is>
-          <t>Chipotle Mexican Grill</t>
+          <t>Patties Express</t>
         </is>
       </c>
       <c r="G50" t="inlineStr">
@@ -2134,15 +2134,15 @@
       </c>
       <c r="B51" t="inlineStr">
         <is>
-          <t>2026-07-08</t>
+          <t>2026-07-15</t>
         </is>
       </c>
       <c r="C51" t="n">
-        <v>6.72</v>
+        <v>6.6</v>
       </c>
       <c r="D51" t="inlineStr">
         <is>
-          <t>Food &amp; Dining</t>
+          <t>Transportation</t>
         </is>
       </c>
       <c r="E51" t="inlineStr">
@@ -2152,7 +2152,7 @@
       </c>
       <c r="F51" t="inlineStr">
         <is>
-          <t>Mos Mos Bakery</t>
+          <t>Presto</t>
         </is>
       </c>
       <c r="G51" t="inlineStr">
@@ -2167,11 +2167,11 @@
       </c>
       <c r="B52" t="inlineStr">
         <is>
-          <t>2026-07-08</t>
+          <t>2026-07-15</t>
         </is>
       </c>
       <c r="C52" t="n">
-        <v>2.51</v>
+        <v>7.91</v>
       </c>
       <c r="D52" t="inlineStr">
         <is>
@@ -2185,7 +2185,7 @@
       </c>
       <c r="F52" t="inlineStr">
         <is>
-          <t>Patties Express</t>
+          <t>Zen Kyoto</t>
         </is>
       </c>
       <c r="G52" t="inlineStr">
@@ -2200,15 +2200,15 @@
       </c>
       <c r="B53" t="inlineStr">
         <is>
-          <t>2026-07-08</t>
+          <t>2026-07-14</t>
         </is>
       </c>
       <c r="C53" t="n">
-        <v>6.6</v>
+        <v>38.15</v>
       </c>
       <c r="D53" t="inlineStr">
         <is>
-          <t>Transportation</t>
+          <t>Utilities &amp; Bills</t>
         </is>
       </c>
       <c r="E53" t="inlineStr">
@@ -2218,7 +2218,7 @@
       </c>
       <c r="F53" t="inlineStr">
         <is>
-          <t>Presto</t>
+          <t>Aviva General Insurance</t>
         </is>
       </c>
       <c r="G53" t="inlineStr">
@@ -2233,11 +2233,11 @@
       </c>
       <c r="B54" t="inlineStr">
         <is>
-          <t>2026-07-08</t>
+          <t>2026-07-14</t>
         </is>
       </c>
       <c r="C54" t="n">
-        <v>19.21</v>
+        <v>25.98</v>
       </c>
       <c r="D54" t="inlineStr">
         <is>
@@ -2251,7 +2251,7 @@
       </c>
       <c r="F54" t="inlineStr">
         <is>
-          <t>Sultans Mediterranean Grill</t>
+          <t>Domino's Pizza</t>
         </is>
       </c>
       <c r="G54" t="inlineStr">
@@ -2266,11 +2266,11 @@
       </c>
       <c r="B55" t="inlineStr">
         <is>
-          <t>2026-07-07</t>
+          <t>2026-07-13</t>
         </is>
       </c>
       <c r="C55" t="n">
-        <v>78.3</v>
+        <v>31.63</v>
       </c>
       <c r="D55" t="inlineStr">
         <is>
@@ -2299,15 +2299,15 @@
       </c>
       <c r="B56" t="inlineStr">
         <is>
-          <t>2026-07-07</t>
+          <t>2026-07-13</t>
         </is>
       </c>
       <c r="C56" t="n">
-        <v>8.359999999999999</v>
+        <v>13.56</v>
       </c>
       <c r="D56" t="inlineStr">
         <is>
-          <t>Transportation</t>
+          <t>Food &amp; Dining</t>
         </is>
       </c>
       <c r="E56" t="inlineStr">
@@ -2317,7 +2317,7 @@
       </c>
       <c r="F56" t="inlineStr">
         <is>
-          <t>Lyft</t>
+          <t>La Diperie</t>
         </is>
       </c>
       <c r="G56" t="inlineStr">
@@ -2332,15 +2332,15 @@
       </c>
       <c r="B57" t="inlineStr">
         <is>
-          <t>2026-07-07</t>
+          <t>2026-07-12</t>
         </is>
       </c>
       <c r="C57" t="n">
-        <v>6.72</v>
+        <v>11.65</v>
       </c>
       <c r="D57" t="inlineStr">
         <is>
-          <t>Food &amp; Dining</t>
+          <t>Shopping &amp; Retail</t>
         </is>
       </c>
       <c r="E57" t="inlineStr">
@@ -2350,7 +2350,7 @@
       </c>
       <c r="F57" t="inlineStr">
         <is>
-          <t>Mos Mos Bakery</t>
+          <t>Amazon</t>
         </is>
       </c>
       <c r="G57" t="inlineStr">
@@ -2365,11 +2365,11 @@
       </c>
       <c r="B58" t="inlineStr">
         <is>
-          <t>2026-07-07</t>
+          <t>2026-07-12</t>
         </is>
       </c>
       <c r="C58" t="n">
-        <v>5.02</v>
+        <v>45.96</v>
       </c>
       <c r="D58" t="inlineStr">
         <is>
@@ -2383,7 +2383,7 @@
       </c>
       <c r="F58" t="inlineStr">
         <is>
-          <t>Patties Express</t>
+          <t>Domino's Pizza</t>
         </is>
       </c>
       <c r="G58" t="inlineStr">
@@ -2398,15 +2398,15 @@
       </c>
       <c r="B59" t="inlineStr">
         <is>
-          <t>2026-07-07</t>
+          <t>2026-07-11</t>
         </is>
       </c>
       <c r="C59" t="n">
-        <v>3.3</v>
+        <v>29.88</v>
       </c>
       <c r="D59" t="inlineStr">
         <is>
-          <t>Transportation</t>
+          <t>Food &amp; Dining</t>
         </is>
       </c>
       <c r="E59" t="inlineStr">
@@ -2416,7 +2416,7 @@
       </c>
       <c r="F59" t="inlineStr">
         <is>
-          <t>Presto</t>
+          <t>McDonald's</t>
         </is>
       </c>
       <c r="G59" t="inlineStr">
@@ -2431,15 +2431,15 @@
       </c>
       <c r="B60" t="inlineStr">
         <is>
-          <t>2026-07-07</t>
+          <t>2026-07-11</t>
         </is>
       </c>
       <c r="C60" t="n">
-        <v>158.2</v>
+        <v>5.24</v>
       </c>
       <c r="D60" t="inlineStr">
         <is>
-          <t>Shopping &amp; Retail</t>
+          <t>Food &amp; Dining</t>
         </is>
       </c>
       <c r="E60" t="inlineStr">
@@ -2449,7 +2449,7 @@
       </c>
       <c r="F60" t="inlineStr">
         <is>
-          <t>JD Sports</t>
+          <t>Mount Molson Dairy Bar</t>
         </is>
       </c>
       <c r="G60" t="inlineStr">
@@ -2464,15 +2464,15 @@
       </c>
       <c r="B61" t="inlineStr">
         <is>
-          <t>2026-07-07</t>
+          <t>2026-07-10</t>
         </is>
       </c>
       <c r="C61" t="n">
-        <v>21.71</v>
+        <v>40.38</v>
       </c>
       <c r="D61" t="inlineStr">
         <is>
-          <t>Transportation</t>
+          <t>Food &amp; Dining</t>
         </is>
       </c>
       <c r="E61" t="inlineStr">
@@ -2482,7 +2482,7 @@
       </c>
       <c r="F61" t="inlineStr">
         <is>
-          <t>Union Station Toronto</t>
+          <t>Domino's Pizza</t>
         </is>
       </c>
       <c r="G61" t="inlineStr">
@@ -2497,11 +2497,11 @@
       </c>
       <c r="B62" t="inlineStr">
         <is>
-          <t>2026-07-07</t>
+          <t>2026-07-10</t>
         </is>
       </c>
       <c r="C62" t="n">
-        <v>39.14</v>
+        <v>3.15</v>
       </c>
       <c r="D62" t="inlineStr">
         <is>
@@ -2515,7 +2515,7 @@
       </c>
       <c r="F62" t="inlineStr">
         <is>
-          <t>Uber Eats</t>
+          <t>McDonald's</t>
         </is>
       </c>
       <c r="G62" t="inlineStr">
@@ -2530,15 +2530,15 @@
       </c>
       <c r="B63" t="inlineStr">
         <is>
-          <t>2026-07-07</t>
+          <t>2026-07-10</t>
         </is>
       </c>
       <c r="C63" t="n">
-        <v>38.39</v>
+        <v>18.16</v>
       </c>
       <c r="D63" t="inlineStr">
         <is>
-          <t>Shopping &amp; Retail</t>
+          <t>Food &amp; Dining</t>
         </is>
       </c>
       <c r="E63" t="inlineStr">
@@ -2548,7 +2548,7 @@
       </c>
       <c r="F63" t="inlineStr">
         <is>
-          <t>Winners</t>
+          <t>McDonald's</t>
         </is>
       </c>
       <c r="G63" t="inlineStr">
@@ -2563,15 +2563,15 @@
       </c>
       <c r="B64" t="inlineStr">
         <is>
-          <t>2026-07-05</t>
+          <t>2026-07-10</t>
         </is>
       </c>
       <c r="C64" t="n">
-        <v>63.39</v>
+        <v>20.54</v>
       </c>
       <c r="D64" t="inlineStr">
         <is>
-          <t>Food &amp; Dining</t>
+          <t>Shopping &amp; Retail</t>
         </is>
       </c>
       <c r="E64" t="inlineStr">
@@ -2581,7 +2581,7 @@
       </c>
       <c r="F64" t="inlineStr">
         <is>
-          <t>JOEY King Street</t>
+          <t>Walmart</t>
         </is>
       </c>
       <c r="G64" t="inlineStr">
@@ -2596,11 +2596,11 @@
       </c>
       <c r="B65" t="inlineStr">
         <is>
-          <t>2026-07-05</t>
+          <t>2026-07-09</t>
         </is>
       </c>
       <c r="C65" t="n">
-        <v>14.75</v>
+        <v>22.2</v>
       </c>
       <c r="D65" t="inlineStr">
         <is>
@@ -2614,7 +2614,7 @@
       </c>
       <c r="F65" t="inlineStr">
         <is>
-          <t>Uncle Tetsu's Japanese Cheesecake</t>
+          <t>Chipotle Mexican Grill</t>
         </is>
       </c>
       <c r="G65" t="inlineStr">
@@ -2629,15 +2629,15 @@
       </c>
       <c r="B66" t="inlineStr">
         <is>
-          <t>2026-07-04</t>
+          <t>2026-07-08</t>
         </is>
       </c>
       <c r="C66" t="n">
-        <v>55.94</v>
+        <v>6.72</v>
       </c>
       <c r="D66" t="inlineStr">
         <is>
-          <t>Entertainment &amp; Leisure</t>
+          <t>Food &amp; Dining</t>
         </is>
       </c>
       <c r="E66" t="inlineStr">
@@ -2647,7 +2647,7 @@
       </c>
       <c r="F66" t="inlineStr">
         <is>
-          <t>Cineplex</t>
+          <t>Mos Mos Bakery</t>
         </is>
       </c>
       <c r="G66" t="inlineStr">
@@ -2662,11 +2662,11 @@
       </c>
       <c r="B67" t="inlineStr">
         <is>
-          <t>2026-07-04</t>
+          <t>2026-07-08</t>
         </is>
       </c>
       <c r="C67" t="n">
-        <v>20.57</v>
+        <v>2.51</v>
       </c>
       <c r="D67" t="inlineStr">
         <is>
@@ -2680,7 +2680,7 @@
       </c>
       <c r="F67" t="inlineStr">
         <is>
-          <t>Uber Eats</t>
+          <t>Patties Express</t>
         </is>
       </c>
       <c r="G67" t="inlineStr">
@@ -2695,15 +2695,15 @@
       </c>
       <c r="B68" t="inlineStr">
         <is>
-          <t>2026-07-03</t>
+          <t>2026-07-08</t>
         </is>
       </c>
       <c r="C68" t="n">
-        <v>6.72</v>
+        <v>6.6</v>
       </c>
       <c r="D68" t="inlineStr">
         <is>
-          <t>Food &amp; Dining</t>
+          <t>Transportation</t>
         </is>
       </c>
       <c r="E68" t="inlineStr">
@@ -2713,7 +2713,7 @@
       </c>
       <c r="F68" t="inlineStr">
         <is>
-          <t>Mos Mos Bakery</t>
+          <t>Presto</t>
         </is>
       </c>
       <c r="G68" t="inlineStr">
@@ -2728,15 +2728,15 @@
       </c>
       <c r="B69" t="inlineStr">
         <is>
-          <t>2026-07-03</t>
+          <t>2026-07-08</t>
         </is>
       </c>
       <c r="C69" t="n">
-        <v>3.3</v>
+        <v>19.21</v>
       </c>
       <c r="D69" t="inlineStr">
         <is>
-          <t>Transportation</t>
+          <t>Food &amp; Dining</t>
         </is>
       </c>
       <c r="E69" t="inlineStr">
@@ -2746,7 +2746,7 @@
       </c>
       <c r="F69" t="inlineStr">
         <is>
-          <t>Presto</t>
+          <t>Sultans Mediterranean Grill</t>
         </is>
       </c>
       <c r="G69" t="inlineStr">
@@ -2761,15 +2761,15 @@
       </c>
       <c r="B70" t="inlineStr">
         <is>
-          <t>2026-07-03</t>
+          <t>2026-07-07</t>
         </is>
       </c>
       <c r="C70" t="n">
-        <v>35.35</v>
+        <v>78.3</v>
       </c>
       <c r="D70" t="inlineStr">
         <is>
-          <t>Food &amp; Dining</t>
+          <t>Shopping &amp; Retail</t>
         </is>
       </c>
       <c r="E70" t="inlineStr">
@@ -2779,7 +2779,7 @@
       </c>
       <c r="F70" t="inlineStr">
         <is>
-          <t>Uber Eats</t>
+          <t>Amazon</t>
         </is>
       </c>
       <c r="G70" t="inlineStr">
@@ -2794,15 +2794,15 @@
       </c>
       <c r="B71" t="inlineStr">
         <is>
-          <t>2026-07-02</t>
+          <t>2026-07-07</t>
         </is>
       </c>
       <c r="C71" t="n">
-        <v>18.08</v>
+        <v>8.359999999999999</v>
       </c>
       <c r="D71" t="inlineStr">
         <is>
-          <t>Food &amp; Dining</t>
+          <t>Transportation</t>
         </is>
       </c>
       <c r="E71" t="inlineStr">
@@ -2812,7 +2812,7 @@
       </c>
       <c r="F71" t="inlineStr">
         <is>
-          <t>Mailo's</t>
+          <t>Lyft</t>
         </is>
       </c>
       <c r="G71" t="inlineStr">
@@ -2827,15 +2827,15 @@
       </c>
       <c r="B72" t="inlineStr">
         <is>
-          <t>2026-06-30</t>
+          <t>2026-07-07</t>
         </is>
       </c>
       <c r="C72" t="n">
-        <v>1.46</v>
+        <v>6.72</v>
       </c>
       <c r="D72" t="inlineStr">
         <is>
-          <t>Entertainment &amp; Leisure</t>
+          <t>Food &amp; Dining</t>
         </is>
       </c>
       <c r="E72" t="inlineStr">
@@ -2845,7 +2845,7 @@
       </c>
       <c r="F72" t="inlineStr">
         <is>
-          <t>Apple</t>
+          <t>Mos Mos Bakery</t>
         </is>
       </c>
       <c r="G72" t="inlineStr">
@@ -2860,11 +2860,11 @@
       </c>
       <c r="B73" t="inlineStr">
         <is>
-          <t>2026-06-29</t>
+          <t>2026-07-07</t>
         </is>
       </c>
       <c r="C73" t="n">
-        <v>25.94</v>
+        <v>5.02</v>
       </c>
       <c r="D73" t="inlineStr">
         <is>
@@ -2878,7 +2878,7 @@
       </c>
       <c r="F73" t="inlineStr">
         <is>
-          <t>Dave's Hot Chicken</t>
+          <t>Patties Express</t>
         </is>
       </c>
       <c r="G73" t="inlineStr">
@@ -2893,15 +2893,15 @@
       </c>
       <c r="B74" t="inlineStr">
         <is>
-          <t>2026-06-29</t>
+          <t>2026-07-07</t>
         </is>
       </c>
       <c r="C74" t="n">
-        <v>2.51</v>
+        <v>3.3</v>
       </c>
       <c r="D74" t="inlineStr">
         <is>
-          <t>Food &amp; Dining</t>
+          <t>Transportation</t>
         </is>
       </c>
       <c r="E74" t="inlineStr">
@@ -2911,7 +2911,7 @@
       </c>
       <c r="F74" t="inlineStr">
         <is>
-          <t>Patties Express</t>
+          <t>Presto</t>
         </is>
       </c>
       <c r="G74" t="inlineStr">
@@ -2926,15 +2926,15 @@
       </c>
       <c r="B75" t="inlineStr">
         <is>
-          <t>2026-06-29</t>
+          <t>2026-07-07</t>
         </is>
       </c>
       <c r="C75" t="n">
-        <v>3.3</v>
+        <v>158.2</v>
       </c>
       <c r="D75" t="inlineStr">
         <is>
-          <t>Transportation</t>
+          <t>Shopping &amp; Retail</t>
         </is>
       </c>
       <c r="E75" t="inlineStr">
@@ -2944,7 +2944,7 @@
       </c>
       <c r="F75" t="inlineStr">
         <is>
-          <t>Presto</t>
+          <t>JD Sports</t>
         </is>
       </c>
       <c r="G75" t="inlineStr">
@@ -2959,15 +2959,15 @@
       </c>
       <c r="B76" t="inlineStr">
         <is>
-          <t>2026-06-29</t>
+          <t>2026-07-07</t>
         </is>
       </c>
       <c r="C76" t="n">
-        <v>75.63</v>
+        <v>21.71</v>
       </c>
       <c r="D76" t="inlineStr">
         <is>
-          <t>Shopping &amp; Retail</t>
+          <t>Transportation</t>
         </is>
       </c>
       <c r="E76" t="inlineStr">
@@ -2977,7 +2977,7 @@
       </c>
       <c r="F76" t="inlineStr">
         <is>
-          <t>Walmart</t>
+          <t>Union Station Toronto</t>
         </is>
       </c>
       <c r="G76" t="inlineStr">
@@ -2992,11 +2992,11 @@
       </c>
       <c r="B77" t="inlineStr">
         <is>
-          <t>2026-06-28</t>
+          <t>2026-07-07</t>
         </is>
       </c>
       <c r="C77" t="n">
-        <v>25.99</v>
+        <v>39.14</v>
       </c>
       <c r="D77" t="inlineStr">
         <is>
@@ -3010,7 +3010,7 @@
       </c>
       <c r="F77" t="inlineStr">
         <is>
-          <t>Chipotle Mexican Grill</t>
+          <t>Uber Eats</t>
         </is>
       </c>
       <c r="G77" t="inlineStr">
@@ -3025,15 +3025,15 @@
       </c>
       <c r="B78" t="inlineStr">
         <is>
-          <t>2026-06-28</t>
+          <t>2026-07-07</t>
         </is>
       </c>
       <c r="C78" t="n">
-        <v>16.39</v>
+        <v>38.39</v>
       </c>
       <c r="D78" t="inlineStr">
         <is>
-          <t>Food &amp; Dining</t>
+          <t>Shopping &amp; Retail</t>
         </is>
       </c>
       <c r="E78" t="inlineStr">
@@ -3043,7 +3043,7 @@
       </c>
       <c r="F78" t="inlineStr">
         <is>
-          <t>Prince Street Pizza</t>
+          <t>Winners</t>
         </is>
       </c>
       <c r="G78" t="inlineStr">
@@ -3058,11 +3058,11 @@
       </c>
       <c r="B79" t="inlineStr">
         <is>
-          <t>2026-06-27</t>
+          <t>2026-07-05</t>
         </is>
       </c>
       <c r="C79" t="n">
-        <v>7.97</v>
+        <v>63.39</v>
       </c>
       <c r="D79" t="inlineStr">
         <is>
@@ -3076,7 +3076,7 @@
       </c>
       <c r="F79" t="inlineStr">
         <is>
-          <t>Balzac's Coffee Roasters</t>
+          <t>JOEY King Street</t>
         </is>
       </c>
       <c r="G79" t="inlineStr">
@@ -3091,15 +3091,15 @@
       </c>
       <c r="B80" t="inlineStr">
         <is>
-          <t>2026-06-27</t>
+          <t>2026-07-05</t>
         </is>
       </c>
       <c r="C80" t="n">
-        <v>42.09</v>
+        <v>14.75</v>
       </c>
       <c r="D80" t="inlineStr">
         <is>
-          <t>Shopping &amp; Retail</t>
+          <t>Food &amp; Dining</t>
         </is>
       </c>
       <c r="E80" t="inlineStr">
@@ -3109,7 +3109,7 @@
       </c>
       <c r="F80" t="inlineStr">
         <is>
-          <t>Dollarama</t>
+          <t>Uncle Tetsu's Japanese Cheesecake</t>
         </is>
       </c>
       <c r="G80" t="inlineStr">
@@ -3124,28 +3124,523 @@
       </c>
       <c r="B81" t="inlineStr">
         <is>
+          <t>2026-07-04</t>
+        </is>
+      </c>
+      <c r="C81" t="n">
+        <v>55.94</v>
+      </c>
+      <c r="D81" t="inlineStr">
+        <is>
+          <t>Entertainment &amp; Leisure</t>
+        </is>
+      </c>
+      <c r="E81" t="inlineStr">
+        <is>
+          <t>Amex Card</t>
+        </is>
+      </c>
+      <c r="F81" t="inlineStr">
+        <is>
+          <t>Cineplex</t>
+        </is>
+      </c>
+      <c r="G81" t="inlineStr">
+        <is>
+          <t>2026-08-14 00:04</t>
+        </is>
+      </c>
+    </row>
+    <row r="82">
+      <c r="A82" t="n">
+        <v>81</v>
+      </c>
+      <c r="B82" t="inlineStr">
+        <is>
+          <t>2026-07-04</t>
+        </is>
+      </c>
+      <c r="C82" t="n">
+        <v>20.57</v>
+      </c>
+      <c r="D82" t="inlineStr">
+        <is>
+          <t>Food &amp; Dining</t>
+        </is>
+      </c>
+      <c r="E82" t="inlineStr">
+        <is>
+          <t>Amex Card</t>
+        </is>
+      </c>
+      <c r="F82" t="inlineStr">
+        <is>
+          <t>Uber Eats</t>
+        </is>
+      </c>
+      <c r="G82" t="inlineStr">
+        <is>
+          <t>2026-08-14 00:04</t>
+        </is>
+      </c>
+    </row>
+    <row r="83">
+      <c r="A83" t="n">
+        <v>82</v>
+      </c>
+      <c r="B83" t="inlineStr">
+        <is>
+          <t>2026-07-03</t>
+        </is>
+      </c>
+      <c r="C83" t="n">
+        <v>6.72</v>
+      </c>
+      <c r="D83" t="inlineStr">
+        <is>
+          <t>Food &amp; Dining</t>
+        </is>
+      </c>
+      <c r="E83" t="inlineStr">
+        <is>
+          <t>Amex Card</t>
+        </is>
+      </c>
+      <c r="F83" t="inlineStr">
+        <is>
+          <t>Mos Mos Bakery</t>
+        </is>
+      </c>
+      <c r="G83" t="inlineStr">
+        <is>
+          <t>2026-08-14 00:04</t>
+        </is>
+      </c>
+    </row>
+    <row r="84">
+      <c r="A84" t="n">
+        <v>83</v>
+      </c>
+      <c r="B84" t="inlineStr">
+        <is>
+          <t>2026-07-03</t>
+        </is>
+      </c>
+      <c r="C84" t="n">
+        <v>3.3</v>
+      </c>
+      <c r="D84" t="inlineStr">
+        <is>
+          <t>Transportation</t>
+        </is>
+      </c>
+      <c r="E84" t="inlineStr">
+        <is>
+          <t>Amex Card</t>
+        </is>
+      </c>
+      <c r="F84" t="inlineStr">
+        <is>
+          <t>Presto</t>
+        </is>
+      </c>
+      <c r="G84" t="inlineStr">
+        <is>
+          <t>2026-08-14 00:04</t>
+        </is>
+      </c>
+    </row>
+    <row r="85">
+      <c r="A85" t="n">
+        <v>84</v>
+      </c>
+      <c r="B85" t="inlineStr">
+        <is>
+          <t>2026-07-03</t>
+        </is>
+      </c>
+      <c r="C85" t="n">
+        <v>35.35</v>
+      </c>
+      <c r="D85" t="inlineStr">
+        <is>
+          <t>Food &amp; Dining</t>
+        </is>
+      </c>
+      <c r="E85" t="inlineStr">
+        <is>
+          <t>Amex Card</t>
+        </is>
+      </c>
+      <c r="F85" t="inlineStr">
+        <is>
+          <t>Uber Eats</t>
+        </is>
+      </c>
+      <c r="G85" t="inlineStr">
+        <is>
+          <t>2026-08-14 00:04</t>
+        </is>
+      </c>
+    </row>
+    <row r="86">
+      <c r="A86" t="n">
+        <v>85</v>
+      </c>
+      <c r="B86" t="inlineStr">
+        <is>
+          <t>2026-07-02</t>
+        </is>
+      </c>
+      <c r="C86" t="n">
+        <v>18.08</v>
+      </c>
+      <c r="D86" t="inlineStr">
+        <is>
+          <t>Food &amp; Dining</t>
+        </is>
+      </c>
+      <c r="E86" t="inlineStr">
+        <is>
+          <t>Amex Card</t>
+        </is>
+      </c>
+      <c r="F86" t="inlineStr">
+        <is>
+          <t>Mailo's</t>
+        </is>
+      </c>
+      <c r="G86" t="inlineStr">
+        <is>
+          <t>2026-08-14 00:04</t>
+        </is>
+      </c>
+    </row>
+    <row r="87">
+      <c r="A87" t="n">
+        <v>86</v>
+      </c>
+      <c r="B87" t="inlineStr">
+        <is>
+          <t>2026-06-30</t>
+        </is>
+      </c>
+      <c r="C87" t="n">
+        <v>1.46</v>
+      </c>
+      <c r="D87" t="inlineStr">
+        <is>
+          <t>Entertainment &amp; Leisure</t>
+        </is>
+      </c>
+      <c r="E87" t="inlineStr">
+        <is>
+          <t>Amex Card</t>
+        </is>
+      </c>
+      <c r="F87" t="inlineStr">
+        <is>
+          <t>Apple</t>
+        </is>
+      </c>
+      <c r="G87" t="inlineStr">
+        <is>
+          <t>2026-08-14 00:04</t>
+        </is>
+      </c>
+    </row>
+    <row r="88">
+      <c r="A88" t="n">
+        <v>87</v>
+      </c>
+      <c r="B88" t="inlineStr">
+        <is>
+          <t>2026-06-29</t>
+        </is>
+      </c>
+      <c r="C88" t="n">
+        <v>25.94</v>
+      </c>
+      <c r="D88" t="inlineStr">
+        <is>
+          <t>Food &amp; Dining</t>
+        </is>
+      </c>
+      <c r="E88" t="inlineStr">
+        <is>
+          <t>Amex Card</t>
+        </is>
+      </c>
+      <c r="F88" t="inlineStr">
+        <is>
+          <t>Dave's Hot Chicken</t>
+        </is>
+      </c>
+      <c r="G88" t="inlineStr">
+        <is>
+          <t>2026-08-14 00:04</t>
+        </is>
+      </c>
+    </row>
+    <row r="89">
+      <c r="A89" t="n">
+        <v>88</v>
+      </c>
+      <c r="B89" t="inlineStr">
+        <is>
+          <t>2026-06-29</t>
+        </is>
+      </c>
+      <c r="C89" t="n">
+        <v>2.51</v>
+      </c>
+      <c r="D89" t="inlineStr">
+        <is>
+          <t>Food &amp; Dining</t>
+        </is>
+      </c>
+      <c r="E89" t="inlineStr">
+        <is>
+          <t>Amex Card</t>
+        </is>
+      </c>
+      <c r="F89" t="inlineStr">
+        <is>
+          <t>Patties Express</t>
+        </is>
+      </c>
+      <c r="G89" t="inlineStr">
+        <is>
+          <t>2026-08-14 00:04</t>
+        </is>
+      </c>
+    </row>
+    <row r="90">
+      <c r="A90" t="n">
+        <v>89</v>
+      </c>
+      <c r="B90" t="inlineStr">
+        <is>
+          <t>2026-06-29</t>
+        </is>
+      </c>
+      <c r="C90" t="n">
+        <v>3.3</v>
+      </c>
+      <c r="D90" t="inlineStr">
+        <is>
+          <t>Transportation</t>
+        </is>
+      </c>
+      <c r="E90" t="inlineStr">
+        <is>
+          <t>Amex Card</t>
+        </is>
+      </c>
+      <c r="F90" t="inlineStr">
+        <is>
+          <t>Presto</t>
+        </is>
+      </c>
+      <c r="G90" t="inlineStr">
+        <is>
+          <t>2026-08-14 00:04</t>
+        </is>
+      </c>
+    </row>
+    <row r="91">
+      <c r="A91" t="n">
+        <v>90</v>
+      </c>
+      <c r="B91" t="inlineStr">
+        <is>
+          <t>2026-06-29</t>
+        </is>
+      </c>
+      <c r="C91" t="n">
+        <v>75.63</v>
+      </c>
+      <c r="D91" t="inlineStr">
+        <is>
+          <t>Shopping &amp; Retail</t>
+        </is>
+      </c>
+      <c r="E91" t="inlineStr">
+        <is>
+          <t>Amex Card</t>
+        </is>
+      </c>
+      <c r="F91" t="inlineStr">
+        <is>
+          <t>Walmart</t>
+        </is>
+      </c>
+      <c r="G91" t="inlineStr">
+        <is>
+          <t>2026-08-14 00:04</t>
+        </is>
+      </c>
+    </row>
+    <row r="92">
+      <c r="A92" t="n">
+        <v>91</v>
+      </c>
+      <c r="B92" t="inlineStr">
+        <is>
+          <t>2026-06-28</t>
+        </is>
+      </c>
+      <c r="C92" t="n">
+        <v>25.99</v>
+      </c>
+      <c r="D92" t="inlineStr">
+        <is>
+          <t>Food &amp; Dining</t>
+        </is>
+      </c>
+      <c r="E92" t="inlineStr">
+        <is>
+          <t>Amex Card</t>
+        </is>
+      </c>
+      <c r="F92" t="inlineStr">
+        <is>
+          <t>Chipotle Mexican Grill</t>
+        </is>
+      </c>
+      <c r="G92" t="inlineStr">
+        <is>
+          <t>2026-08-14 00:04</t>
+        </is>
+      </c>
+    </row>
+    <row r="93">
+      <c r="A93" t="n">
+        <v>92</v>
+      </c>
+      <c r="B93" t="inlineStr">
+        <is>
+          <t>2026-06-28</t>
+        </is>
+      </c>
+      <c r="C93" t="n">
+        <v>16.39</v>
+      </c>
+      <c r="D93" t="inlineStr">
+        <is>
+          <t>Food &amp; Dining</t>
+        </is>
+      </c>
+      <c r="E93" t="inlineStr">
+        <is>
+          <t>Amex Card</t>
+        </is>
+      </c>
+      <c r="F93" t="inlineStr">
+        <is>
+          <t>Prince Street Pizza</t>
+        </is>
+      </c>
+      <c r="G93" t="inlineStr">
+        <is>
+          <t>2026-08-14 00:04</t>
+        </is>
+      </c>
+    </row>
+    <row r="94">
+      <c r="A94" t="n">
+        <v>93</v>
+      </c>
+      <c r="B94" t="inlineStr">
+        <is>
+          <t>2026-06-27</t>
+        </is>
+      </c>
+      <c r="C94" t="n">
+        <v>7.97</v>
+      </c>
+      <c r="D94" t="inlineStr">
+        <is>
+          <t>Food &amp; Dining</t>
+        </is>
+      </c>
+      <c r="E94" t="inlineStr">
+        <is>
+          <t>Amex Card</t>
+        </is>
+      </c>
+      <c r="F94" t="inlineStr">
+        <is>
+          <t>Balzac's Coffee Roasters</t>
+        </is>
+      </c>
+      <c r="G94" t="inlineStr">
+        <is>
+          <t>2026-08-14 00:04</t>
+        </is>
+      </c>
+    </row>
+    <row r="95">
+      <c r="A95" t="n">
+        <v>94</v>
+      </c>
+      <c r="B95" t="inlineStr">
+        <is>
+          <t>2026-06-27</t>
+        </is>
+      </c>
+      <c r="C95" t="n">
+        <v>42.09</v>
+      </c>
+      <c r="D95" t="inlineStr">
+        <is>
+          <t>Shopping &amp; Retail</t>
+        </is>
+      </c>
+      <c r="E95" t="inlineStr">
+        <is>
+          <t>Amex Card</t>
+        </is>
+      </c>
+      <c r="F95" t="inlineStr">
+        <is>
+          <t>Dollarama</t>
+        </is>
+      </c>
+      <c r="G95" t="inlineStr">
+        <is>
+          <t>2026-08-14 00:04</t>
+        </is>
+      </c>
+    </row>
+    <row r="96">
+      <c r="A96" t="n">
+        <v>95</v>
+      </c>
+      <c r="B96" t="inlineStr">
+        <is>
           <t>2026-06-26</t>
         </is>
       </c>
-      <c r="C81" t="n">
+      <c r="C96" t="n">
         <v>18.08</v>
       </c>
-      <c r="D81" t="inlineStr">
-        <is>
-          <t>Food &amp; Dining</t>
-        </is>
-      </c>
-      <c r="E81" t="inlineStr">
-        <is>
-          <t>Amex Card</t>
-        </is>
-      </c>
-      <c r="F81" t="inlineStr">
+      <c r="D96" t="inlineStr">
+        <is>
+          <t>Food &amp; Dining</t>
+        </is>
+      </c>
+      <c r="E96" t="inlineStr">
+        <is>
+          <t>Amex Card</t>
+        </is>
+      </c>
+      <c r="F96" t="inlineStr">
         <is>
           <t>Mailo's</t>
         </is>
       </c>
-      <c r="G81" t="inlineStr">
+      <c r="G96" t="inlineStr">
         <is>
           <t>2026-08-14 00:04</t>
         </is>
@@ -3198,7 +3693,7 @@
       </c>
       <c r="C2" t="inlineStr">
         <is>
-          <t>2026-08-13 23:33</t>
+          <t>2026-08-14 00:00</t>
         </is>
       </c>
     </row>
@@ -3213,7 +3708,7 @@
       </c>
       <c r="C3" t="inlineStr">
         <is>
-          <t>2026-08-13 23:33</t>
+          <t>2026-08-14 00:00</t>
         </is>
       </c>
     </row>
@@ -3228,7 +3723,7 @@
       </c>
       <c r="C4" t="inlineStr">
         <is>
-          <t>2026-08-13 23:33</t>
+          <t>2026-08-14 00:00</t>
         </is>
       </c>
     </row>
@@ -3243,7 +3738,7 @@
       </c>
       <c r="C5" t="inlineStr">
         <is>
-          <t>2026-08-13 23:33</t>
+          <t>2026-08-14 00:00</t>
         </is>
       </c>
     </row>
@@ -3258,7 +3753,7 @@
       </c>
       <c r="C6" t="inlineStr">
         <is>
-          <t>2026-08-13 23:33</t>
+          <t>2026-08-14 00:00</t>
         </is>
       </c>
     </row>
@@ -3273,7 +3768,7 @@
       </c>
       <c r="C7" t="inlineStr">
         <is>
-          <t>2026-08-13 23:33</t>
+          <t>2026-08-14 00:00</t>
         </is>
       </c>
     </row>
@@ -3288,7 +3783,7 @@
       </c>
       <c r="C8" t="inlineStr">
         <is>
-          <t>2026-08-13 23:33</t>
+          <t>2026-08-14 00:00</t>
         </is>
       </c>
     </row>
@@ -3303,7 +3798,7 @@
       </c>
       <c r="C9" t="inlineStr">
         <is>
-          <t>2026-08-13 23:33</t>
+          <t>2026-08-14 00:00</t>
         </is>
       </c>
     </row>
@@ -3318,7 +3813,7 @@
       </c>
       <c r="C10" t="inlineStr">
         <is>
-          <t>2026-08-13 23:33</t>
+          <t>2026-08-14 00:00</t>
         </is>
       </c>
     </row>
@@ -3333,7 +3828,7 @@
       </c>
       <c r="C11" t="inlineStr">
         <is>
-          <t>2026-08-13 23:33</t>
+          <t>2026-08-14 00:00</t>
         </is>
       </c>
     </row>
@@ -3348,7 +3843,7 @@
       </c>
       <c r="C12" t="inlineStr">
         <is>
-          <t>2026-08-13 23:33</t>
+          <t>2026-08-14 00:00</t>
         </is>
       </c>
     </row>
@@ -3363,7 +3858,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:C12"/>
+  <dimension ref="A1:C13"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="27" customWidth="1" min="1" max="1"/>
@@ -3561,15 +4056,32 @@
     <row r="12">
       <c r="A12" t="inlineStr">
         <is>
+          <t>Refunds &amp; Credits</t>
+        </is>
+      </c>
+      <c r="B12" t="inlineStr">
+        <is>
+          <t>#10B981</t>
+        </is>
+      </c>
+      <c r="C12" t="inlineStr">
+        <is>
+          <t>rotate-left</t>
+        </is>
+      </c>
+    </row>
+    <row r="13">
+      <c r="A13" t="inlineStr">
+        <is>
           <t>Miscellaneous</t>
         </is>
       </c>
-      <c r="B12" t="inlineStr">
+      <c r="B13" t="inlineStr">
         <is>
           <t>#64748B</t>
         </is>
       </c>
-      <c r="C12" t="inlineStr">
+      <c r="C13" t="inlineStr">
         <is>
           <t>tags</t>
         </is>

</xml_diff>